<commit_message>
Add NO/FB logic, Type column, Option rule fix, and skill reference
- run.py: full rewrite — Type column (NC→NO=False, NO→NO=True), VLV_W_FB/FB_OPN_EN/FB_CLS_EN from FB rows, Option rule forces only ENABLE/EXIST=False, auto-discovered tag map with unquoted Options unit fix, COLS_PER_FAM=16
- EnvoraSiemens_Skill.md: new domain reference file (DB format, CW bits, business rules, gotchas)
- prompt.txt, wishList.md, DesignStructure.md, PROJECT_LEARNINGS.md: corrected NO logic (NC→False, NO→True) and updated all rules
- Re-ran all 5 products (Brew/Clara/CR/KR/PP); updated comparison xlsx and updated db files

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testLBB.xlsx
+++ b/testLBB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SETUMHNE\Downloads\myLearning\gitPlayGround\PlayGround\TestDB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\Agentic World\TestDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6BC3075-9EB6-47A2-9FD5-D283D546DD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF99A034-B823-44A1-A719-A31EABF5B0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2440DDF5-C456-4655-B2B4-B11D9C3116FA}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{2440DDF5-C456-4655-B2B4-B11D9C3116FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -62,27 +62,51 @@
   <commentList>
     <comment ref="E24" authorId="0" shapeId="0" xr:uid="{C9784531-5C6D-44EC-AB65-162B1CE3680D}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    True</t>
+    False</t>
+        </r>
       </text>
     </comment>
     <comment ref="E30" authorId="1" shapeId="0" xr:uid="{71BB7FBC-F32F-4C72-9332-1C81A6EC2304}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    False</t>
+    True</t>
+        </r>
       </text>
     </comment>
     <comment ref="B110" authorId="2" shapeId="0" xr:uid="{73D4B7F6-243F-4FF2-99C8-413E3B588F2F}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative tag labels:
 PIT220-1 / PIT221-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="F110" authorId="3" shapeId="0" xr:uid="{ACEAC60E-563F-4328-B54F-2D31DA895568}">
@@ -311,11 +335,19 @@
     </comment>
     <comment ref="B116" authorId="4" shapeId="0" xr:uid="{4608516B-34DA-4E87-85F1-345F80F368D2}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative tag labels:
 PIT221-1 / PIT220-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="S116" authorId="3" shapeId="0" xr:uid="{32126A50-CE7D-4FF2-ADF3-AC79E3BFC8D7}">
@@ -376,11 +408,19 @@
     </comment>
     <comment ref="B130" authorId="5" shapeId="0" xr:uid="{37D13463-1186-4BC6-8059-F81F589B8465}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative tag labels:
 PCV220-1 / PCV221-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="F130" authorId="3" shapeId="0" xr:uid="{A163B90D-1EF5-443F-899F-87AE8DB0F188}">
@@ -609,11 +649,19 @@
     </comment>
     <comment ref="B132" authorId="6" shapeId="0" xr:uid="{330CC50C-0FF1-4C20-92A7-B1A460F72FE0}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative tag labels:
 PCV221-1 / PCV220-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="S132" authorId="3" shapeId="0" xr:uid="{22150A06-9848-4929-8ED5-23E9E8AE01F0}">
@@ -674,11 +722,19 @@
     </comment>
     <comment ref="B139" authorId="7" shapeId="0" xr:uid="{C128BBFA-0A9E-4E10-9DCF-02753B677457}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative labels:
 ST740/ST741</t>
+        </r>
       </text>
     </comment>
     <comment ref="F139" authorId="3" shapeId="0" xr:uid="{71DF5CC9-8C1C-486E-B5BB-3BCC7CA84727}">
@@ -935,11 +991,19 @@
     </comment>
     <comment ref="B187" authorId="8" shapeId="0" xr:uid="{FAC71602-7205-4D4E-A8A7-63E13947D7F3}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative tag labels:
 LS422b / LS423</t>
+        </r>
       </text>
     </comment>
     <comment ref="J187" authorId="3" shapeId="0" xr:uid="{7BE8016D-9A39-41FB-B16C-9D5E1B3F75EA}">
@@ -986,11 +1050,19 @@
     </comment>
     <comment ref="B212" authorId="9" shapeId="0" xr:uid="{4A8C6723-E87B-4DCF-BC82-3EEAFFA13634}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative labels:
 YT750/YT752</t>
+        </r>
       </text>
     </comment>
     <comment ref="F212" authorId="3" shapeId="0" xr:uid="{7A748396-5D90-45A2-BCDA-09E9D00EB824}">
@@ -1247,11 +1319,19 @@
     </comment>
     <comment ref="B214" authorId="10" shapeId="0" xr:uid="{932F2D4C-D793-48A0-8BED-5F38FC3D7DAF}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative labels:
 PT375-1/PT376-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="G214" authorId="3" shapeId="0" xr:uid="{A7A9E8D1-727E-4B93-BDEB-E67DFF623450}">
@@ -1494,36 +1574,68 @@
     </comment>
     <comment ref="B218" authorId="11" shapeId="0" xr:uid="{E1E2F944-CF9F-4061-9330-99AC06440908}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative sensors, same PIW:
 TT731b/TT733</t>
+        </r>
       </text>
     </comment>
     <comment ref="G218" authorId="12" shapeId="0" xr:uid="{F8073023-E3D6-437F-A368-4B60DA804058}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Sensor: TT733</t>
+        </r>
       </text>
     </comment>
     <comment ref="L218" authorId="13" shapeId="0" xr:uid="{ED46C518-7286-47D1-963D-3F59595A0F45}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Sensor: TT731b</t>
+        </r>
       </text>
     </comment>
     <comment ref="B223" authorId="14" shapeId="0" xr:uid="{FCEB49F4-8B73-4CA2-A393-7AEBAA66145D}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative labels:
 TT410-1/TT412-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="F223" authorId="3" shapeId="0" xr:uid="{3F0AF3B0-2ABB-45F3-8CF9-4442E029B36F}">
@@ -1780,19 +1892,35 @@
     </comment>
     <comment ref="B243" authorId="15" shapeId="0" xr:uid="{C29E9803-A59F-4197-99DC-10131D1A8691}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Old AV635b-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="B248" authorId="16" shapeId="0" xr:uid="{F05B5C03-D80C-44EE-911F-FD4F08369CD1}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative labels:
 AV375-1/AV376-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="F248" authorId="3" shapeId="0" xr:uid="{7EF7BC57-4FCC-448F-8A09-38CD88A5340F}">
@@ -2063,11 +2191,19 @@
     </comment>
     <comment ref="B252" authorId="17" shapeId="0" xr:uid="{6BE60107-F28C-41F1-A623-84DD5A6A045C}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative labels:
 AV441-1/AV630-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="M252" authorId="3" shapeId="0" xr:uid="{6F128C66-A3BA-4965-B079-6A928BE29365}">
@@ -2086,11 +2222,19 @@
     </comment>
     <comment ref="B253" authorId="18" shapeId="0" xr:uid="{573F35F3-86C4-417F-BDB5-9F88836E09BB}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Alfa Laval Offc"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Alternative labels:
 506c/AV372-1</t>
+        </r>
       </text>
     </comment>
     <comment ref="F253" authorId="3" shapeId="0" xr:uid="{68836ADC-7909-428F-90A1-5710219BA6C4}">
@@ -3530,7 +3674,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3577,12 +3721,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -4257,23 +4395,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5555E797-91C5-44FA-95FC-58DB33F30F80}">
   <dimension ref="B1:W401"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="10.75" style="1" customWidth="1"/>
     <col min="3" max="3" width="31.25" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.75" style="1" customWidth="1"/>
-    <col min="5" max="5" width="5.75" style="10" customWidth="1"/>
+    <col min="5" max="5" width="6.5" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="2.25" style="10" customWidth="1"/>
-    <col min="8" max="9" width="2.83203125" style="10" customWidth="1"/>
+    <col min="8" max="9" width="2.875" style="10" customWidth="1"/>
     <col min="10" max="12" width="6.75" style="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="2.58203125" style="10" customWidth="1"/>
-    <col min="16" max="16" width="2.83203125" style="10" customWidth="1"/>
-    <col min="17" max="17" width="2.58203125" style="10" customWidth="1"/>
-    <col min="18" max="22" width="2.83203125" style="10" customWidth="1"/>
-    <col min="23" max="23" width="2.58203125" style="10" customWidth="1"/>
+    <col min="13" max="15" width="2.625" style="10" customWidth="1"/>
+    <col min="16" max="16" width="2.875" style="10" customWidth="1"/>
+    <col min="17" max="17" width="2.625" style="10" customWidth="1"/>
+    <col min="18" max="22" width="2.875" style="10" customWidth="1"/>
+    <col min="23" max="23" width="2.625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" ht="35.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:23" ht="35.25" customHeight="1">
       <c r="D1" s="1" t="s">
         <v>285</v>
       </c>
@@ -4332,7 +4470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="2:23" ht="57" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:23" ht="58.5">
       <c r="B2"/>
       <c r="C2"/>
       <c r="D2"/>
@@ -4392,7 +4530,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="3" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:23">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -4424,7 +4562,7 @@
       <c r="V3" s="12"/>
       <c r="W3" s="12"/>
     </row>
-    <row r="4" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:23">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -4448,7 +4586,7 @@
       <c r="V4" s="13"/>
       <c r="W4" s="13"/>
     </row>
-    <row r="5" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:23">
       <c r="B5" s="4"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -4472,7 +4610,7 @@
       <c r="V5" s="14"/>
       <c r="W5" s="14"/>
     </row>
-    <row r="6" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:23">
       <c r="B6" s="4"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -4496,7 +4634,7 @@
       <c r="V6" s="13"/>
       <c r="W6" s="13"/>
     </row>
-    <row r="7" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:23">
       <c r="B7" s="4" t="s">
         <v>1</v>
       </c>
@@ -4560,7 +4698,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="8" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:23">
       <c r="B8" s="4" t="s">
         <v>2</v>
       </c>
@@ -4620,7 +4758,7 @@
       </c>
       <c r="W8" s="13"/>
     </row>
-    <row r="9" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:23">
       <c r="B9" s="4" t="s">
         <v>3</v>
       </c>
@@ -4680,7 +4818,7 @@
       </c>
       <c r="W9" s="13"/>
     </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:23">
       <c r="B10" s="4" t="s">
         <v>4</v>
       </c>
@@ -4718,7 +4856,7 @@
       </c>
       <c r="W10" s="13"/>
     </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:23">
       <c r="B11" s="4" t="s">
         <v>5</v>
       </c>
@@ -4782,7 +4920,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:23">
       <c r="B12" s="4" t="s">
         <v>6</v>
       </c>
@@ -4846,7 +4984,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="13" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:23">
       <c r="B13" s="4" t="s">
         <v>7</v>
       </c>
@@ -4910,7 +5048,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:23">
       <c r="B14" s="5" t="s">
         <v>8</v>
       </c>
@@ -4938,7 +5076,7 @@
       <c r="V14" s="13"/>
       <c r="W14" s="13"/>
     </row>
-    <row r="15" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:23">
       <c r="B15" s="5" t="s">
         <v>8</v>
       </c>
@@ -4966,7 +5104,7 @@
       <c r="V15" s="13"/>
       <c r="W15" s="13"/>
     </row>
-    <row r="16" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:23">
       <c r="B16" s="4" t="s">
         <v>9</v>
       </c>
@@ -5020,7 +5158,7 @@
       <c r="V16" s="13"/>
       <c r="W16" s="13"/>
     </row>
-    <row r="17" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:23">
       <c r="B17" s="4" t="s">
         <v>10</v>
       </c>
@@ -5078,7 +5216,7 @@
       </c>
       <c r="W17" s="13"/>
     </row>
-    <row r="18" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:23">
       <c r="B18" s="4" t="s">
         <v>11</v>
       </c>
@@ -5122,7 +5260,7 @@
       <c r="V18" s="13"/>
       <c r="W18" s="13"/>
     </row>
-    <row r="19" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:23">
       <c r="B19" s="5" t="s">
         <v>8</v>
       </c>
@@ -5150,7 +5288,7 @@
       <c r="V19" s="13"/>
       <c r="W19" s="13"/>
     </row>
-    <row r="20" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:23">
       <c r="B20" s="5" t="s">
         <v>8</v>
       </c>
@@ -5178,7 +5316,7 @@
       <c r="V20" s="13"/>
       <c r="W20" s="13"/>
     </row>
-    <row r="21" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:23">
       <c r="B21" s="5" t="s">
         <v>8</v>
       </c>
@@ -5206,7 +5344,7 @@
       <c r="V21" s="13"/>
       <c r="W21" s="13"/>
     </row>
-    <row r="22" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:23">
       <c r="B22" s="4" t="s">
         <v>12</v>
       </c>
@@ -5272,7 +5410,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="23" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:23">
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -5296,7 +5434,7 @@
       <c r="V23" s="13"/>
       <c r="W23" s="13"/>
     </row>
-    <row r="24" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:23">
       <c r="B24" s="6" t="s">
         <v>13</v>
       </c>
@@ -5362,7 +5500,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="25" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:23">
       <c r="B25" s="6" t="s">
         <v>13</v>
       </c>
@@ -5428,7 +5566,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="26" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:23">
       <c r="B26" s="6" t="s">
         <v>14</v>
       </c>
@@ -5474,7 +5612,7 @@
       <c r="V26" s="13"/>
       <c r="W26" s="13"/>
     </row>
-    <row r="27" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:23">
       <c r="B27" s="6" t="s">
         <v>14</v>
       </c>
@@ -5520,7 +5658,7 @@
       <c r="V27" s="13"/>
       <c r="W27" s="13"/>
     </row>
-    <row r="28" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:23">
       <c r="B28" s="6" t="s">
         <v>15</v>
       </c>
@@ -5566,7 +5704,7 @@
       <c r="V28" s="13"/>
       <c r="W28" s="13"/>
     </row>
-    <row r="29" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:23">
       <c r="B29" s="6" t="s">
         <v>15</v>
       </c>
@@ -5612,7 +5750,7 @@
       <c r="V29" s="13"/>
       <c r="W29" s="13"/>
     </row>
-    <row r="30" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:23">
       <c r="B30" s="6" t="s">
         <v>16</v>
       </c>
@@ -5656,7 +5794,7 @@
       <c r="V30" s="13"/>
       <c r="W30" s="13"/>
     </row>
-    <row r="31" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:23">
       <c r="B31" s="6" t="s">
         <v>16</v>
       </c>
@@ -5700,7 +5838,7 @@
       <c r="V31" s="13"/>
       <c r="W31" s="13"/>
     </row>
-    <row r="32" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:23">
       <c r="B32" s="6" t="s">
         <v>17</v>
       </c>
@@ -5762,7 +5900,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="33" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:23">
       <c r="B33" s="6" t="s">
         <v>17</v>
       </c>
@@ -5824,7 +5962,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:23">
       <c r="B34" s="6" t="s">
         <v>18</v>
       </c>
@@ -5864,7 +6002,7 @@
       </c>
       <c r="W34" s="13"/>
     </row>
-    <row r="35" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:23">
       <c r="B35" s="6" t="s">
         <v>18</v>
       </c>
@@ -5904,7 +6042,7 @@
       </c>
       <c r="W35" s="13"/>
     </row>
-    <row r="36" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:23">
       <c r="B36" s="6" t="s">
         <v>19</v>
       </c>
@@ -5948,7 +6086,7 @@
       <c r="V36" s="13"/>
       <c r="W36" s="13"/>
     </row>
-    <row r="37" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:23">
       <c r="B37" s="7" t="s">
         <v>19</v>
       </c>
@@ -5992,7 +6130,7 @@
       <c r="V37" s="15"/>
       <c r="W37" s="15"/>
     </row>
-    <row r="38" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:23">
       <c r="B38" s="5" t="s">
         <v>8</v>
       </c>
@@ -6020,7 +6158,7 @@
       <c r="V38" s="13"/>
       <c r="W38" s="13"/>
     </row>
-    <row r="39" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:23">
       <c r="B39" s="5" t="s">
         <v>8</v>
       </c>
@@ -6048,7 +6186,7 @@
       <c r="V39" s="13"/>
       <c r="W39" s="13"/>
     </row>
-    <row r="40" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:23">
       <c r="B40" s="4"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -6072,7 +6210,7 @@
       <c r="V40" s="13"/>
       <c r="W40" s="13"/>
     </row>
-    <row r="41" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:23">
       <c r="B41" s="7" t="s">
         <v>20</v>
       </c>
@@ -6138,7 +6276,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:23">
       <c r="B42" s="6" t="s">
         <v>20</v>
       </c>
@@ -6204,7 +6342,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:23">
       <c r="B43" s="6" t="s">
         <v>21</v>
       </c>
@@ -6270,7 +6408,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="44" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:23">
       <c r="B44" s="6" t="s">
         <v>21</v>
       </c>
@@ -6336,7 +6474,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:23">
       <c r="B45" s="6" t="s">
         <v>22</v>
       </c>
@@ -6402,7 +6540,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:23">
       <c r="B46" s="6" t="s">
         <v>22</v>
       </c>
@@ -6468,7 +6606,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:23">
       <c r="B47" s="6" t="s">
         <v>23</v>
       </c>
@@ -6526,7 +6664,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:23">
       <c r="B48" s="6" t="s">
         <v>23</v>
       </c>
@@ -6584,7 +6722,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="49" spans="2:23">
       <c r="B49" s="6" t="s">
         <v>24</v>
       </c>
@@ -6646,7 +6784,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="50" spans="2:23">
       <c r="B50" s="6" t="s">
         <v>24</v>
       </c>
@@ -6708,7 +6846,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="51" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="51" spans="2:23">
       <c r="B51" s="6" t="s">
         <v>25</v>
       </c>
@@ -6766,7 +6904,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="52" spans="2:23">
       <c r="B52" s="6" t="s">
         <v>25</v>
       </c>
@@ -6824,7 +6962,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="53" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:23">
       <c r="B53" s="6" t="s">
         <v>26</v>
       </c>
@@ -6866,7 +7004,7 @@
       <c r="V53" s="13"/>
       <c r="W53" s="13"/>
     </row>
-    <row r="54" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="54" spans="2:23">
       <c r="B54" s="6" t="s">
         <v>26</v>
       </c>
@@ -6908,7 +7046,7 @@
       <c r="V54" s="13"/>
       <c r="W54" s="13"/>
     </row>
-    <row r="55" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="55" spans="2:23">
       <c r="B55" s="5" t="s">
         <v>8</v>
       </c>
@@ -6936,7 +7074,7 @@
       <c r="V55" s="13"/>
       <c r="W55" s="13"/>
     </row>
-    <row r="56" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="56" spans="2:23">
       <c r="B56" s="5" t="s">
         <v>8</v>
       </c>
@@ -6964,7 +7102,7 @@
       <c r="V56" s="13"/>
       <c r="W56" s="13"/>
     </row>
-    <row r="57" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="57" spans="2:23">
       <c r="B57" s="6"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
@@ -6988,7 +7126,7 @@
       <c r="V57" s="13"/>
       <c r="W57" s="13"/>
     </row>
-    <row r="58" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:23">
       <c r="B58" s="6" t="s">
         <v>27</v>
       </c>
@@ -7032,7 +7170,7 @@
       <c r="V58" s="13"/>
       <c r="W58" s="13"/>
     </row>
-    <row r="59" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:23">
       <c r="B59" s="6" t="s">
         <v>27</v>
       </c>
@@ -7076,7 +7214,7 @@
       <c r="V59" s="13"/>
       <c r="W59" s="13"/>
     </row>
-    <row r="60" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="60" spans="2:23">
       <c r="B60" s="5" t="s">
         <v>8</v>
       </c>
@@ -7104,7 +7242,7 @@
       <c r="V60" s="13"/>
       <c r="W60" s="13"/>
     </row>
-    <row r="61" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:23">
       <c r="B61" s="5" t="s">
         <v>8</v>
       </c>
@@ -7132,7 +7270,7 @@
       <c r="V61" s="13"/>
       <c r="W61" s="13"/>
     </row>
-    <row r="62" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="62" spans="2:23">
       <c r="B62" s="6" t="s">
         <v>28</v>
       </c>
@@ -7190,7 +7328,7 @@
       </c>
       <c r="W62" s="13"/>
     </row>
-    <row r="63" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="63" spans="2:23">
       <c r="B63" s="6" t="s">
         <v>28</v>
       </c>
@@ -7248,7 +7386,7 @@
       </c>
       <c r="W63" s="13"/>
     </row>
-    <row r="64" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:23">
       <c r="B64" s="6" t="s">
         <v>29</v>
       </c>
@@ -7306,7 +7444,7 @@
       </c>
       <c r="W64" s="13"/>
     </row>
-    <row r="65" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="65" spans="2:23">
       <c r="B65" s="6" t="s">
         <v>29</v>
       </c>
@@ -7364,7 +7502,7 @@
       </c>
       <c r="W65" s="13"/>
     </row>
-    <row r="66" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="66" spans="2:23">
       <c r="B66" s="6" t="s">
         <v>30</v>
       </c>
@@ -7404,7 +7542,7 @@
       </c>
       <c r="W66" s="13"/>
     </row>
-    <row r="67" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:23">
       <c r="B67" s="6" t="s">
         <v>30</v>
       </c>
@@ -7444,7 +7582,7 @@
       </c>
       <c r="W67" s="13"/>
     </row>
-    <row r="68" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="68" spans="2:23">
       <c r="B68" s="5" t="s">
         <v>8</v>
       </c>
@@ -7472,7 +7610,7 @@
       <c r="V68" s="13"/>
       <c r="W68" s="13"/>
     </row>
-    <row r="69" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:23">
       <c r="B69" s="5" t="s">
         <v>8</v>
       </c>
@@ -7500,7 +7638,7 @@
       <c r="V69" s="13"/>
       <c r="W69" s="13"/>
     </row>
-    <row r="70" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="70" spans="2:23">
       <c r="B70" s="5" t="s">
         <v>8</v>
       </c>
@@ -7528,7 +7666,7 @@
       <c r="V70" s="13"/>
       <c r="W70" s="13"/>
     </row>
-    <row r="71" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="71" spans="2:23">
       <c r="B71" s="5" t="s">
         <v>8</v>
       </c>
@@ -7556,7 +7694,7 @@
       <c r="V71" s="13"/>
       <c r="W71" s="13"/>
     </row>
-    <row r="72" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:23">
       <c r="B72" s="5" t="s">
         <v>8</v>
       </c>
@@ -7584,7 +7722,7 @@
       <c r="V72" s="13"/>
       <c r="W72" s="13"/>
     </row>
-    <row r="73" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="73" spans="2:23">
       <c r="B73" s="5" t="s">
         <v>8</v>
       </c>
@@ -7612,7 +7750,7 @@
       <c r="V73" s="13"/>
       <c r="W73" s="13"/>
     </row>
-    <row r="74" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:23">
       <c r="B74" s="6"/>
       <c r="C74" s="3"/>
       <c r="D74" s="20"/>
@@ -7636,7 +7774,7 @@
       <c r="V74" s="13"/>
       <c r="W74" s="13"/>
     </row>
-    <row r="75" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:23">
       <c r="B75" s="6" t="s">
         <v>13</v>
       </c>
@@ -7702,7 +7840,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="76" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:23">
       <c r="B76" s="6" t="s">
         <v>14</v>
       </c>
@@ -7748,7 +7886,7 @@
       <c r="V76" s="13"/>
       <c r="W76" s="13"/>
     </row>
-    <row r="77" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="77" spans="2:23">
       <c r="B77" s="6" t="s">
         <v>15</v>
       </c>
@@ -7794,7 +7932,7 @@
       <c r="V77" s="13"/>
       <c r="W77" s="13"/>
     </row>
-    <row r="78" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:23">
       <c r="B78" s="6" t="s">
         <v>16</v>
       </c>
@@ -7838,7 +7976,7 @@
       <c r="V78" s="13"/>
       <c r="W78" s="13"/>
     </row>
-    <row r="79" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="79" spans="2:23">
       <c r="B79" s="6" t="s">
         <v>17</v>
       </c>
@@ -7900,7 +8038,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="80" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="80" spans="2:23">
       <c r="B80" s="6" t="s">
         <v>18</v>
       </c>
@@ -7940,7 +8078,7 @@
       </c>
       <c r="W80" s="13"/>
     </row>
-    <row r="81" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="81" spans="2:23">
       <c r="B81" s="6" t="s">
         <v>19</v>
       </c>
@@ -7984,7 +8122,7 @@
       <c r="V81" s="13"/>
       <c r="W81" s="13"/>
     </row>
-    <row r="82" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="82" spans="2:23">
       <c r="B82" s="5" t="s">
         <v>8</v>
       </c>
@@ -8012,7 +8150,7 @@
       <c r="V82" s="13"/>
       <c r="W82" s="13"/>
     </row>
-    <row r="83" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="83" spans="2:23">
       <c r="B83" s="6" t="s">
         <v>20</v>
       </c>
@@ -8078,7 +8216,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="84" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="84" spans="2:23">
       <c r="B84" s="6" t="s">
         <v>21</v>
       </c>
@@ -8144,7 +8282,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="85" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="85" spans="2:23">
       <c r="B85" s="6" t="s">
         <v>22</v>
       </c>
@@ -8210,7 +8348,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="86" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="86" spans="2:23">
       <c r="B86" s="6" t="s">
         <v>23</v>
       </c>
@@ -8268,7 +8406,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="87" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="87" spans="2:23">
       <c r="B87" s="6" t="s">
         <v>24</v>
       </c>
@@ -8330,7 +8468,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="88" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="88" spans="2:23">
       <c r="B88" s="6" t="s">
         <v>25</v>
       </c>
@@ -8388,7 +8526,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="89" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="89" spans="2:23">
       <c r="B89" s="6" t="s">
         <v>26</v>
       </c>
@@ -8430,7 +8568,7 @@
       <c r="V89" s="13"/>
       <c r="W89" s="13"/>
     </row>
-    <row r="90" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="90" spans="2:23">
       <c r="B90" s="5" t="s">
         <v>8</v>
       </c>
@@ -8458,7 +8596,7 @@
       <c r="V90" s="13"/>
       <c r="W90" s="13"/>
     </row>
-    <row r="91" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="91" spans="2:23">
       <c r="B91" s="6"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
@@ -8482,7 +8620,7 @@
       <c r="V91" s="13"/>
       <c r="W91" s="13"/>
     </row>
-    <row r="92" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="92" spans="2:23">
       <c r="B92" s="6" t="s">
         <v>27</v>
       </c>
@@ -8526,7 +8664,7 @@
       <c r="V92" s="13"/>
       <c r="W92" s="13"/>
     </row>
-    <row r="93" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="93" spans="2:23">
       <c r="B93" s="5" t="s">
         <v>8</v>
       </c>
@@ -8556,7 +8694,7 @@
       <c r="V93" s="13"/>
       <c r="W93" s="13"/>
     </row>
-    <row r="94" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="94" spans="2:23">
       <c r="B94" s="6" t="s">
         <v>28</v>
       </c>
@@ -8614,7 +8752,7 @@
       </c>
       <c r="W94" s="13"/>
     </row>
-    <row r="95" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="95" spans="2:23">
       <c r="B95" s="6" t="s">
         <v>29</v>
       </c>
@@ -8672,7 +8810,7 @@
       </c>
       <c r="W95" s="13"/>
     </row>
-    <row r="96" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="96" spans="2:23">
       <c r="B96" s="6" t="s">
         <v>30</v>
       </c>
@@ -8712,7 +8850,7 @@
       </c>
       <c r="W96" s="13"/>
     </row>
-    <row r="97" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="97" spans="2:23">
       <c r="B97" s="5" t="s">
         <v>8</v>
       </c>
@@ -8740,7 +8878,7 @@
       <c r="V97" s="13"/>
       <c r="W97" s="13"/>
     </row>
-    <row r="98" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="98" spans="2:23">
       <c r="B98" s="5" t="s">
         <v>8</v>
       </c>
@@ -8768,7 +8906,7 @@
       <c r="V98" s="13"/>
       <c r="W98" s="13"/>
     </row>
-    <row r="99" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="99" spans="2:23">
       <c r="B99" s="5" t="s">
         <v>8</v>
       </c>
@@ -8796,7 +8934,7 @@
       <c r="V99" s="13"/>
       <c r="W99" s="13"/>
     </row>
-    <row r="100" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="100" spans="2:23">
       <c r="B100" s="5" t="s">
         <v>8</v>
       </c>
@@ -8824,7 +8962,7 @@
       <c r="V100" s="13"/>
       <c r="W100" s="13"/>
     </row>
-    <row r="101" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="101" spans="2:23">
       <c r="B101" s="4" t="s">
         <v>31</v>
       </c>
@@ -8866,7 +9004,7 @@
       <c r="V101" s="13"/>
       <c r="W101" s="13"/>
     </row>
-    <row r="102" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="102" spans="2:23">
       <c r="B102" s="8" t="s">
         <v>32</v>
       </c>
@@ -8930,7 +9068,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="103" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="103" spans="2:23">
       <c r="B103" s="4" t="s">
         <v>290</v>
       </c>
@@ -8994,7 +9132,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="104" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="104" spans="2:23">
       <c r="B104" s="4" t="s">
         <v>291</v>
       </c>
@@ -9036,7 +9174,7 @@
       <c r="V104" s="13"/>
       <c r="W104" s="13"/>
     </row>
-    <row r="105" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="105" spans="2:23">
       <c r="B105" s="4" t="s">
         <v>292</v>
       </c>
@@ -9100,7 +9238,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="106" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="106" spans="2:23">
       <c r="B106" s="4" t="s">
         <v>33</v>
       </c>
@@ -9164,7 +9302,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="107" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="107" spans="2:23">
       <c r="B107" s="4" t="s">
         <v>34</v>
       </c>
@@ -9192,7 +9330,7 @@
       <c r="V107" s="13"/>
       <c r="W107" s="13"/>
     </row>
-    <row r="108" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="108" spans="2:23">
       <c r="B108" s="4"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
@@ -9216,7 +9354,7 @@
       <c r="V108" s="13"/>
       <c r="W108" s="13"/>
     </row>
-    <row r="109" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="109" spans="2:23">
       <c r="B109" s="4" t="s">
         <v>35</v>
       </c>
@@ -9282,7 +9420,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="110" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="110" spans="2:23">
       <c r="B110" s="4" t="s">
         <v>36</v>
       </c>
@@ -9344,7 +9482,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="111" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="111" spans="2:23">
       <c r="B111" s="4" t="s">
         <v>37</v>
       </c>
@@ -9400,7 +9538,7 @@
       <c r="V111" s="13"/>
       <c r="W111" s="13"/>
     </row>
-    <row r="112" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="112" spans="2:23">
       <c r="B112" s="4" t="s">
         <v>38</v>
       </c>
@@ -9460,7 +9598,7 @@
       </c>
       <c r="W112" s="13"/>
     </row>
-    <row r="113" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="113" spans="2:23">
       <c r="B113" s="4"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
@@ -9484,7 +9622,7 @@
       <c r="V113" s="13"/>
       <c r="W113" s="13"/>
     </row>
-    <row r="114" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="114" spans="2:23">
       <c r="B114" s="4" t="s">
         <v>39</v>
       </c>
@@ -9530,7 +9668,7 @@
       <c r="V114" s="13"/>
       <c r="W114" s="13"/>
     </row>
-    <row r="115" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="115" spans="2:23">
       <c r="B115" s="5" t="s">
         <v>8</v>
       </c>
@@ -9558,7 +9696,7 @@
       <c r="V115" s="13"/>
       <c r="W115" s="13"/>
     </row>
-    <row r="116" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="116" spans="2:23">
       <c r="B116" s="4" t="s">
         <v>40</v>
       </c>
@@ -9598,7 +9736,7 @@
       </c>
       <c r="W116" s="13"/>
     </row>
-    <row r="117" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="117" spans="2:23">
       <c r="B117" s="4" t="s">
         <v>41</v>
       </c>
@@ -9630,7 +9768,7 @@
       <c r="V117" s="13"/>
       <c r="W117" s="13"/>
     </row>
-    <row r="118" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="118" spans="2:23">
       <c r="B118" s="4"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
@@ -9654,7 +9792,7 @@
       <c r="V118" s="13"/>
       <c r="W118" s="13"/>
     </row>
-    <row r="119" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="119" spans="2:23">
       <c r="B119" s="4" t="s">
         <v>42</v>
       </c>
@@ -9720,7 +9858,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="120" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="120" spans="2:23">
       <c r="B120" s="4" t="s">
         <v>43</v>
       </c>
@@ -9778,7 +9916,7 @@
       </c>
       <c r="W120" s="13"/>
     </row>
-    <row r="121" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="121" spans="2:23">
       <c r="B121" s="4" t="s">
         <v>44</v>
       </c>
@@ -9836,7 +9974,7 @@
       </c>
       <c r="W121" s="13"/>
     </row>
-    <row r="122" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="122" spans="2:23">
       <c r="B122" s="4" t="s">
         <v>45</v>
       </c>
@@ -9882,7 +10020,7 @@
       <c r="V122" s="13"/>
       <c r="W122" s="13"/>
     </row>
-    <row r="123" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="123" spans="2:23">
       <c r="B123" s="4"/>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
@@ -9906,7 +10044,7 @@
       <c r="V123" s="13"/>
       <c r="W123" s="13"/>
     </row>
-    <row r="124" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="124" spans="2:23">
       <c r="B124" s="4" t="s">
         <v>46</v>
       </c>
@@ -9936,7 +10074,7 @@
       <c r="V124" s="13"/>
       <c r="W124" s="13"/>
     </row>
-    <row r="125" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="125" spans="2:23">
       <c r="B125" s="4" t="s">
         <v>47</v>
       </c>
@@ -9968,7 +10106,7 @@
       <c r="V125" s="13"/>
       <c r="W125" s="13"/>
     </row>
-    <row r="126" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="126" spans="2:23">
       <c r="B126" s="4" t="s">
         <v>48</v>
       </c>
@@ -10036,7 +10174,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="127" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="127" spans="2:23">
       <c r="B127" s="5" t="s">
         <v>8</v>
       </c>
@@ -10066,7 +10204,7 @@
       <c r="V127" s="13"/>
       <c r="W127" s="13"/>
     </row>
-    <row r="128" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="128" spans="2:23">
       <c r="B128" s="4"/>
       <c r="C128" s="3"/>
       <c r="D128" s="19"/>
@@ -10090,7 +10228,7 @@
       <c r="V128" s="13"/>
       <c r="W128" s="13"/>
     </row>
-    <row r="129" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="129" spans="2:23">
       <c r="B129" s="4" t="s">
         <v>49</v>
       </c>
@@ -10156,7 +10294,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="130" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="130" spans="2:23">
       <c r="B130" s="4" t="s">
         <v>50</v>
       </c>
@@ -10218,7 +10356,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="131" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="131" spans="2:23">
       <c r="B131" s="4" t="s">
         <v>51</v>
       </c>
@@ -10284,7 +10422,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="132" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="132" spans="2:23">
       <c r="B132" s="4" t="s">
         <v>52</v>
       </c>
@@ -10322,7 +10460,7 @@
       </c>
       <c r="W132" s="13"/>
     </row>
-    <row r="133" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="133" spans="2:23">
       <c r="B133" s="4"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
@@ -10346,7 +10484,7 @@
       <c r="V133" s="13"/>
       <c r="W133" s="13"/>
     </row>
-    <row r="134" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="134" spans="2:23">
       <c r="B134" s="4" t="s">
         <v>53</v>
       </c>
@@ -10392,7 +10530,7 @@
       <c r="V134" s="13"/>
       <c r="W134" s="13"/>
     </row>
-    <row r="135" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="135" spans="2:23">
       <c r="B135" s="4" t="s">
         <v>54</v>
       </c>
@@ -10438,7 +10576,7 @@
       <c r="V135" s="13"/>
       <c r="W135" s="13"/>
     </row>
-    <row r="136" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="136" spans="2:23">
       <c r="B136" s="4" t="s">
         <v>55</v>
       </c>
@@ -10484,7 +10622,7 @@
       <c r="V136" s="13"/>
       <c r="W136" s="13"/>
     </row>
-    <row r="137" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="137" spans="2:23">
       <c r="B137" s="4" t="s">
         <v>56</v>
       </c>
@@ -10552,7 +10690,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="138" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="138" spans="2:23">
       <c r="B138" s="4"/>
       <c r="C138" s="3"/>
       <c r="D138" s="3"/>
@@ -10576,7 +10714,7 @@
       <c r="V138" s="13"/>
       <c r="W138" s="13"/>
     </row>
-    <row r="139" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="139" spans="2:23">
       <c r="B139" s="4" t="s">
         <v>57</v>
       </c>
@@ -10640,7 +10778,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="140" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="140" spans="2:23">
       <c r="B140" s="4"/>
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
@@ -10664,7 +10802,7 @@
       <c r="V140" s="13"/>
       <c r="W140" s="13"/>
     </row>
-    <row r="141" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="141" spans="2:23">
       <c r="B141" s="4" t="s">
         <v>58</v>
       </c>
@@ -10696,7 +10834,7 @@
       <c r="V141" s="14"/>
       <c r="W141" s="14"/>
     </row>
-    <row r="142" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="142" spans="2:23">
       <c r="B142" s="4"/>
       <c r="C142" s="3"/>
       <c r="D142" s="3"/>
@@ -10720,7 +10858,7 @@
       <c r="V142" s="13"/>
       <c r="W142" s="13"/>
     </row>
-    <row r="143" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="143" spans="2:23">
       <c r="B143" s="4" t="s">
         <v>59</v>
       </c>
@@ -10784,7 +10922,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="144" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="144" spans="2:23">
       <c r="B144" s="4" t="s">
         <v>60</v>
       </c>
@@ -10848,7 +10986,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="145" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="145" spans="2:23">
       <c r="B145" s="4" t="s">
         <v>61</v>
       </c>
@@ -10912,7 +11050,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="146" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="146" spans="2:23">
       <c r="B146" s="4" t="s">
         <v>62</v>
       </c>
@@ -10976,7 +11114,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="147" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="147" spans="2:23">
       <c r="B147" s="4" t="s">
         <v>63</v>
       </c>
@@ -11040,7 +11178,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="148" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="148" spans="2:23">
       <c r="B148" s="4" t="s">
         <v>64</v>
       </c>
@@ -11100,7 +11238,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="149" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="149" spans="2:23">
       <c r="B149" s="4" t="s">
         <v>65</v>
       </c>
@@ -11166,7 +11304,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="150" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="150" spans="2:23">
       <c r="B150" s="4" t="s">
         <v>66</v>
       </c>
@@ -11198,7 +11336,7 @@
       <c r="V150" s="13"/>
       <c r="W150" s="13"/>
     </row>
-    <row r="151" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="151" spans="2:23">
       <c r="B151" s="4" t="s">
         <v>67</v>
       </c>
@@ -11230,7 +11368,7 @@
       <c r="V151" s="13"/>
       <c r="W151" s="13"/>
     </row>
-    <row r="152" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="152" spans="2:23">
       <c r="B152" s="5" t="s">
         <v>8</v>
       </c>
@@ -11258,7 +11396,7 @@
       <c r="V152" s="13"/>
       <c r="W152" s="13"/>
     </row>
-    <row r="153" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="153" spans="2:23">
       <c r="B153" s="4" t="s">
         <v>68</v>
       </c>
@@ -11322,7 +11460,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="154" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="154" spans="2:23">
       <c r="B154" s="4" t="s">
         <v>68</v>
       </c>
@@ -11386,7 +11524,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="155" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="155" spans="2:23">
       <c r="B155" s="4" t="s">
         <v>69</v>
       </c>
@@ -11452,7 +11590,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="156" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="156" spans="2:23">
       <c r="B156" s="4" t="s">
         <v>69</v>
       </c>
@@ -11518,7 +11656,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="157" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="157" spans="2:23">
       <c r="B157" s="5" t="s">
         <v>8</v>
       </c>
@@ -11546,7 +11684,7 @@
       <c r="V157" s="13"/>
       <c r="W157" s="13"/>
     </row>
-    <row r="158" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="158" spans="2:23">
       <c r="B158" s="5" t="s">
         <v>8</v>
       </c>
@@ -11574,7 +11712,7 @@
       <c r="V158" s="13"/>
       <c r="W158" s="13"/>
     </row>
-    <row r="159" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="159" spans="2:23">
       <c r="B159" s="4"/>
       <c r="C159" s="3"/>
       <c r="D159" s="3"/>
@@ -11598,7 +11736,7 @@
       <c r="V159" s="13"/>
       <c r="W159" s="13"/>
     </row>
-    <row r="160" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="160" spans="2:23">
       <c r="B160" s="4" t="s">
         <v>70</v>
       </c>
@@ -11632,7 +11770,7 @@
       <c r="V160" s="13"/>
       <c r="W160" s="13"/>
     </row>
-    <row r="161" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="161" spans="2:23">
       <c r="B161" s="4" t="s">
         <v>70</v>
       </c>
@@ -11666,7 +11804,7 @@
       <c r="V161" s="13"/>
       <c r="W161" s="13"/>
     </row>
-    <row r="162" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="162" spans="2:23">
       <c r="B162" s="4" t="s">
         <v>71</v>
       </c>
@@ -11710,7 +11848,7 @@
       <c r="V162" s="13"/>
       <c r="W162" s="13"/>
     </row>
-    <row r="163" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="163" spans="2:23">
       <c r="B163" s="4" t="s">
         <v>71</v>
       </c>
@@ -11754,7 +11892,7 @@
       <c r="V163" s="13"/>
       <c r="W163" s="13"/>
     </row>
-    <row r="164" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="164" spans="2:23">
       <c r="B164" s="4" t="s">
         <v>72</v>
       </c>
@@ -11810,7 +11948,7 @@
       </c>
       <c r="W164" s="13"/>
     </row>
-    <row r="165" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="165" spans="2:23">
       <c r="B165" s="4" t="s">
         <v>72</v>
       </c>
@@ -11866,7 +12004,7 @@
       </c>
       <c r="W165" s="13"/>
     </row>
-    <row r="166" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="166" spans="2:23">
       <c r="B166" s="4" t="s">
         <v>73</v>
       </c>
@@ -11932,7 +12070,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="167" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="167" spans="2:23">
       <c r="B167" s="4" t="s">
         <v>73</v>
       </c>
@@ -11998,7 +12136,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="168" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="168" spans="2:23">
       <c r="B168" s="4" t="s">
         <v>74</v>
       </c>
@@ -12042,7 +12180,7 @@
       <c r="V168" s="13"/>
       <c r="W168" s="13"/>
     </row>
-    <row r="169" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="169" spans="2:23">
       <c r="B169" s="4" t="s">
         <v>74</v>
       </c>
@@ -12086,7 +12224,7 @@
       <c r="V169" s="13"/>
       <c r="W169" s="13"/>
     </row>
-    <row r="170" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="170" spans="2:23">
       <c r="B170" s="5" t="s">
         <v>8</v>
       </c>
@@ -12114,7 +12252,7 @@
       <c r="V170" s="13"/>
       <c r="W170" s="13"/>
     </row>
-    <row r="171" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="171" spans="2:23">
       <c r="B171" s="5" t="s">
         <v>8</v>
       </c>
@@ -12142,7 +12280,7 @@
       <c r="V171" s="13"/>
       <c r="W171" s="13"/>
     </row>
-    <row r="172" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="172" spans="2:23">
       <c r="B172" s="5" t="s">
         <v>8</v>
       </c>
@@ -12170,7 +12308,7 @@
       <c r="V172" s="13"/>
       <c r="W172" s="13"/>
     </row>
-    <row r="173" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="173" spans="2:23">
       <c r="B173" s="5" t="s">
         <v>8</v>
       </c>
@@ -12198,7 +12336,7 @@
       <c r="V173" s="13"/>
       <c r="W173" s="13"/>
     </row>
-    <row r="174" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="174" spans="2:23">
       <c r="B174" s="5" t="s">
         <v>8</v>
       </c>
@@ -12226,7 +12364,7 @@
       <c r="V174" s="13"/>
       <c r="W174" s="13"/>
     </row>
-    <row r="175" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="175" spans="2:23">
       <c r="B175" s="5" t="s">
         <v>8</v>
       </c>
@@ -12254,7 +12392,7 @@
       <c r="V175" s="13"/>
       <c r="W175" s="13"/>
     </row>
-    <row r="176" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="176" spans="2:23">
       <c r="B176" s="4"/>
       <c r="C176" s="3"/>
       <c r="D176" s="3"/>
@@ -12278,7 +12416,7 @@
       <c r="V176" s="13"/>
       <c r="W176" s="13"/>
     </row>
-    <row r="177" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="177" spans="2:23">
       <c r="B177" s="4" t="s">
         <v>75</v>
       </c>
@@ -12322,7 +12460,7 @@
       <c r="V177" s="13"/>
       <c r="W177" s="13"/>
     </row>
-    <row r="178" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="178" spans="2:23">
       <c r="B178" s="4" t="s">
         <v>76</v>
       </c>
@@ -12366,7 +12504,7 @@
       <c r="V178" s="13"/>
       <c r="W178" s="13"/>
     </row>
-    <row r="179" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="179" spans="2:23">
       <c r="B179" s="4" t="s">
         <v>77</v>
       </c>
@@ -12410,7 +12548,7 @@
       <c r="V179" s="13"/>
       <c r="W179" s="13"/>
     </row>
-    <row r="180" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="180" spans="2:23">
       <c r="B180" s="4" t="s">
         <v>78</v>
       </c>
@@ -12454,7 +12592,7 @@
       <c r="V180" s="13"/>
       <c r="W180" s="13"/>
     </row>
-    <row r="181" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="181" spans="2:23">
       <c r="B181" s="5" t="s">
         <v>8</v>
       </c>
@@ -12482,7 +12620,7 @@
       <c r="V181" s="13"/>
       <c r="W181" s="13"/>
     </row>
-    <row r="182" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="182" spans="2:23">
       <c r="B182" s="5" t="s">
         <v>8</v>
       </c>
@@ -12510,7 +12648,7 @@
       <c r="V182" s="13"/>
       <c r="W182" s="13"/>
     </row>
-    <row r="183" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="183" spans="2:23">
       <c r="B183" s="4" t="s">
         <v>79</v>
       </c>
@@ -12544,7 +12682,7 @@
       <c r="V183" s="13"/>
       <c r="W183" s="13"/>
     </row>
-    <row r="184" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="184" spans="2:23">
       <c r="B184" s="4" t="s">
         <v>80</v>
       </c>
@@ -12578,7 +12716,7 @@
       <c r="V184" s="13"/>
       <c r="W184" s="13"/>
     </row>
-    <row r="185" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="185" spans="2:23">
       <c r="B185" s="4" t="s">
         <v>81</v>
       </c>
@@ -12612,7 +12750,7 @@
       <c r="V185" s="13"/>
       <c r="W185" s="13"/>
     </row>
-    <row r="186" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="186" spans="2:23">
       <c r="B186" s="4" t="s">
         <v>82</v>
       </c>
@@ -12646,7 +12784,7 @@
       <c r="V186" s="13"/>
       <c r="W186" s="13"/>
     </row>
-    <row r="187" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="187" spans="2:23">
       <c r="B187" s="4" t="s">
         <v>83</v>
       </c>
@@ -12682,7 +12820,7 @@
       <c r="V187" s="13"/>
       <c r="W187" s="13"/>
     </row>
-    <row r="188" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="188" spans="2:23">
       <c r="B188" s="4" t="s">
         <v>84</v>
       </c>
@@ -12716,7 +12854,7 @@
       <c r="V188" s="13"/>
       <c r="W188" s="13"/>
     </row>
-    <row r="189" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="189" spans="2:23">
       <c r="B189" s="4" t="s">
         <v>85</v>
       </c>
@@ -12748,7 +12886,7 @@
       <c r="V189" s="13"/>
       <c r="W189" s="13"/>
     </row>
-    <row r="190" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="190" spans="2:23">
       <c r="B190" s="5" t="s">
         <v>8</v>
       </c>
@@ -12776,7 +12914,7 @@
       <c r="V190" s="13"/>
       <c r="W190" s="13"/>
     </row>
-    <row r="191" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="191" spans="2:23">
       <c r="B191" s="5" t="s">
         <v>8</v>
       </c>
@@ -12804,7 +12942,7 @@
       <c r="V191" s="13"/>
       <c r="W191" s="13"/>
     </row>
-    <row r="192" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="192" spans="2:23">
       <c r="B192" s="5" t="s">
         <v>8</v>
       </c>
@@ -12832,7 +12970,7 @@
       <c r="V192" s="13"/>
       <c r="W192" s="13"/>
     </row>
-    <row r="193" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="193" spans="2:23">
       <c r="B193" s="4"/>
       <c r="C193" s="3"/>
       <c r="D193" s="3"/>
@@ -12856,7 +12994,7 @@
       <c r="V193" s="13"/>
       <c r="W193" s="13"/>
     </row>
-    <row r="194" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="194" spans="2:23">
       <c r="B194" s="4" t="s">
         <v>68</v>
       </c>
@@ -12920,7 +13058,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="195" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="195" spans="2:23">
       <c r="B195" s="4" t="s">
         <v>68</v>
       </c>
@@ -12984,7 +13122,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="196" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="196" spans="2:23">
       <c r="B196" s="4" t="s">
         <v>69</v>
       </c>
@@ -13050,7 +13188,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="197" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="197" spans="2:23">
       <c r="B197" s="4" t="s">
         <v>70</v>
       </c>
@@ -13084,7 +13222,7 @@
       <c r="V197" s="13"/>
       <c r="W197" s="13"/>
     </row>
-    <row r="198" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="198" spans="2:23">
       <c r="B198" s="4" t="s">
         <v>71</v>
       </c>
@@ -13128,7 +13266,7 @@
       <c r="V198" s="13"/>
       <c r="W198" s="13"/>
     </row>
-    <row r="199" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="199" spans="2:23">
       <c r="B199" s="4" t="s">
         <v>72</v>
       </c>
@@ -13184,7 +13322,7 @@
       </c>
       <c r="W199" s="13"/>
     </row>
-    <row r="200" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="200" spans="2:23">
       <c r="B200" s="4" t="s">
         <v>73</v>
       </c>
@@ -13250,7 +13388,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="201" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="201" spans="2:23">
       <c r="B201" s="4" t="s">
         <v>73</v>
       </c>
@@ -13316,7 +13454,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="202" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="202" spans="2:23">
       <c r="B202" s="4" t="s">
         <v>74</v>
       </c>
@@ -13360,7 +13498,7 @@
       <c r="V202" s="13"/>
       <c r="W202" s="13"/>
     </row>
-    <row r="203" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="203" spans="2:23">
       <c r="B203" s="5" t="s">
         <v>8</v>
       </c>
@@ -13388,7 +13526,7 @@
       <c r="V203" s="13"/>
       <c r="W203" s="13"/>
     </row>
-    <row r="204" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="204" spans="2:23">
       <c r="B204" s="4" t="s">
         <v>86</v>
       </c>
@@ -13452,7 +13590,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="205" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="205" spans="2:23">
       <c r="B205" s="5" t="s">
         <v>8</v>
       </c>
@@ -13480,7 +13618,7 @@
       <c r="V205" s="13"/>
       <c r="W205" s="13"/>
     </row>
-    <row r="206" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="206" spans="2:23">
       <c r="B206" s="5" t="s">
         <v>8</v>
       </c>
@@ -13508,7 +13646,7 @@
       <c r="V206" s="13"/>
       <c r="W206" s="13"/>
     </row>
-    <row r="207" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="207" spans="2:23">
       <c r="B207" s="5" t="s">
         <v>8</v>
       </c>
@@ -13536,7 +13674,7 @@
       <c r="V207" s="13"/>
       <c r="W207" s="13"/>
     </row>
-    <row r="208" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="208" spans="2:23">
       <c r="B208" s="5" t="s">
         <v>8</v>
       </c>
@@ -13564,7 +13702,7 @@
       <c r="V208" s="13"/>
       <c r="W208" s="13"/>
     </row>
-    <row r="209" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="209" spans="2:23">
       <c r="B209" s="5" t="s">
         <v>8</v>
       </c>
@@ -13592,7 +13730,7 @@
       <c r="V209" s="13"/>
       <c r="W209" s="13"/>
     </row>
-    <row r="210" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="210" spans="2:23">
       <c r="B210" s="4"/>
       <c r="C210" s="3"/>
       <c r="D210" s="3"/>
@@ -13616,7 +13754,7 @@
       <c r="V210" s="13"/>
       <c r="W210" s="13"/>
     </row>
-    <row r="211" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="211" spans="2:23">
       <c r="B211" s="4" t="s">
         <v>87</v>
       </c>
@@ -13682,7 +13820,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="212" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="212" spans="2:23">
       <c r="B212" s="4" t="s">
         <v>88</v>
       </c>
@@ -13748,7 +13886,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="213" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="213" spans="2:23">
       <c r="B213" s="4" t="s">
         <v>89</v>
       </c>
@@ -13784,7 +13922,7 @@
       <c r="V213" s="13"/>
       <c r="W213" s="13"/>
     </row>
-    <row r="214" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="214" spans="2:23">
       <c r="B214" s="4" t="s">
         <v>90</v>
       </c>
@@ -13842,7 +13980,7 @@
       </c>
       <c r="W214" s="13"/>
     </row>
-    <row r="215" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="215" spans="2:23">
       <c r="B215" s="4"/>
       <c r="C215" s="3"/>
       <c r="D215" s="3"/>
@@ -13866,7 +14004,7 @@
       <c r="V215" s="13"/>
       <c r="W215" s="13"/>
     </row>
-    <row r="216" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="216" spans="2:23">
       <c r="B216" s="4" t="s">
         <v>91</v>
       </c>
@@ -13902,7 +14040,7 @@
       <c r="V216" s="13"/>
       <c r="W216" s="13"/>
     </row>
-    <row r="217" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="217" spans="2:23">
       <c r="B217" s="4" t="s">
         <v>92</v>
       </c>
@@ -13966,7 +14104,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="218" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="218" spans="2:23">
       <c r="B218" s="4" t="s">
         <v>93</v>
       </c>
@@ -14026,7 +14164,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="219" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="219" spans="2:23">
       <c r="B219" s="4" t="s">
         <v>94</v>
       </c>
@@ -14092,7 +14230,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="220" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="220" spans="2:23">
       <c r="B220" s="4" t="s">
         <v>95</v>
       </c>
@@ -14128,7 +14266,7 @@
       <c r="V220" s="13"/>
       <c r="W220" s="13"/>
     </row>
-    <row r="221" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="221" spans="2:23">
       <c r="B221" s="4" t="s">
         <v>96</v>
       </c>
@@ -14164,7 +14302,7 @@
       <c r="V221" s="13"/>
       <c r="W221" s="13"/>
     </row>
-    <row r="222" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="222" spans="2:23">
       <c r="B222" s="4" t="s">
         <v>97</v>
       </c>
@@ -14202,7 +14340,7 @@
       <c r="V222" s="13"/>
       <c r="W222" s="13"/>
     </row>
-    <row r="223" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="223" spans="2:23">
       <c r="B223" s="4" t="s">
         <v>98</v>
       </c>
@@ -14270,7 +14408,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="224" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="224" spans="2:23">
       <c r="B224" s="4"/>
       <c r="C224" s="3"/>
       <c r="D224" s="3"/>
@@ -14294,7 +14432,7 @@
       <c r="V224" s="13"/>
       <c r="W224" s="13"/>
     </row>
-    <row r="225" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="225" spans="2:23">
       <c r="B225" s="4" t="s">
         <v>68</v>
       </c>
@@ -14360,7 +14498,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="226" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="226" spans="2:23">
       <c r="B226" s="4" t="s">
         <v>73</v>
       </c>
@@ -14428,7 +14566,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="227" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="227" spans="2:23">
       <c r="B227" s="5" t="s">
         <v>8</v>
       </c>
@@ -14458,7 +14596,7 @@
       <c r="V227" s="13"/>
       <c r="W227" s="13"/>
     </row>
-    <row r="228" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="228" spans="2:23">
       <c r="B228" s="5" t="s">
         <v>8</v>
       </c>
@@ -14488,7 +14626,7 @@
       <c r="V228" s="13"/>
       <c r="W228" s="13"/>
     </row>
-    <row r="229" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="229" spans="2:23">
       <c r="B229" s="4"/>
       <c r="C229" s="3"/>
       <c r="D229" s="3"/>
@@ -14512,7 +14650,7 @@
       <c r="V229" s="13"/>
       <c r="W229" s="13"/>
     </row>
-    <row r="230" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="230" spans="2:23">
       <c r="B230" s="4"/>
       <c r="C230" s="3" t="s">
         <v>231</v>
@@ -14554,7 +14692,7 @@
       <c r="V230" s="13"/>
       <c r="W230" s="13"/>
     </row>
-    <row r="231" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="231" spans="2:23">
       <c r="B231" s="4"/>
       <c r="C231" s="3" t="s">
         <v>232</v>
@@ -14596,7 +14734,7 @@
       <c r="V231" s="13"/>
       <c r="W231" s="13"/>
     </row>
-    <row r="232" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="232" spans="2:23">
       <c r="B232" s="4"/>
       <c r="C232" s="3"/>
       <c r="D232" s="3"/>
@@ -14620,7 +14758,7 @@
       <c r="V232" s="13"/>
       <c r="W232" s="13"/>
     </row>
-    <row r="233" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="233" spans="2:23">
       <c r="B233" s="4" t="s">
         <v>99</v>
       </c>
@@ -14664,7 +14802,7 @@
       <c r="V233" s="13"/>
       <c r="W233" s="13"/>
     </row>
-    <row r="234" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="234" spans="2:23">
       <c r="B234" s="4" t="s">
         <v>100</v>
       </c>
@@ -14708,7 +14846,7 @@
       <c r="V234" s="13"/>
       <c r="W234" s="13"/>
     </row>
-    <row r="235" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="235" spans="2:23">
       <c r="B235" s="4" t="s">
         <v>101</v>
       </c>
@@ -14752,7 +14890,7 @@
       <c r="V235" s="13"/>
       <c r="W235" s="13"/>
     </row>
-    <row r="236" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="236" spans="2:23">
       <c r="B236" s="5" t="s">
         <v>8</v>
       </c>
@@ -14796,7 +14934,7 @@
       <c r="V236" s="13"/>
       <c r="W236" s="13"/>
     </row>
-    <row r="237" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="237" spans="2:23">
       <c r="B237" s="4"/>
       <c r="C237" s="3"/>
       <c r="D237" s="3"/>
@@ -14820,7 +14958,7 @@
       <c r="V237" s="13"/>
       <c r="W237" s="13"/>
     </row>
-    <row r="238" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="238" spans="2:23">
       <c r="B238" s="4" t="s">
         <v>102</v>
       </c>
@@ -14866,7 +15004,7 @@
       <c r="V238" s="13"/>
       <c r="W238" s="13"/>
     </row>
-    <row r="239" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="239" spans="2:23">
       <c r="B239" s="4" t="s">
         <v>77</v>
       </c>
@@ -14912,7 +15050,7 @@
       <c r="V239" s="13"/>
       <c r="W239" s="13"/>
     </row>
-    <row r="240" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="240" spans="2:23">
       <c r="B240" s="4" t="s">
         <v>103</v>
       </c>
@@ -14958,7 +15096,7 @@
       <c r="V240" s="13"/>
       <c r="W240" s="13"/>
     </row>
-    <row r="241" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="241" spans="2:23">
       <c r="B241" s="4" t="s">
         <v>78</v>
       </c>
@@ -15004,7 +15142,7 @@
       <c r="V241" s="13"/>
       <c r="W241" s="13"/>
     </row>
-    <row r="242" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="242" spans="2:23">
       <c r="B242" s="4"/>
       <c r="C242" s="3"/>
       <c r="D242" s="3"/>
@@ -15028,7 +15166,7 @@
       <c r="V242" s="13"/>
       <c r="W242" s="13"/>
     </row>
-    <row r="243" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="243" spans="2:23">
       <c r="B243" s="4" t="s">
         <v>104</v>
       </c>
@@ -15076,7 +15214,7 @@
       <c r="V243" s="13"/>
       <c r="W243" s="13"/>
     </row>
-    <row r="244" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="244" spans="2:23">
       <c r="B244" s="4" t="s">
         <v>105</v>
       </c>
@@ -15142,7 +15280,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="245" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="245" spans="2:23">
       <c r="B245" s="4" t="s">
         <v>106</v>
       </c>
@@ -15208,7 +15346,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="246" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="246" spans="2:23">
       <c r="B246" s="4" t="s">
         <v>107</v>
       </c>
@@ -15274,7 +15412,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="247" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="247" spans="2:23">
       <c r="B247" s="4" t="s">
         <v>108</v>
       </c>
@@ -15318,7 +15456,7 @@
       <c r="V247" s="13"/>
       <c r="W247" s="13"/>
     </row>
-    <row r="248" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="248" spans="2:23">
       <c r="B248" s="4" t="s">
         <v>109</v>
       </c>
@@ -15384,7 +15522,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="249" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="249" spans="2:23">
       <c r="B249" s="4" t="s">
         <v>110</v>
       </c>
@@ -15450,7 +15588,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="250" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="250" spans="2:23">
       <c r="B250" s="4" t="s">
         <v>111</v>
       </c>
@@ -15512,7 +15650,7 @@
       </c>
       <c r="W250" s="13"/>
     </row>
-    <row r="251" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="251" spans="2:23">
       <c r="B251" s="4" t="s">
         <v>112</v>
       </c>
@@ -15574,7 +15712,7 @@
       </c>
       <c r="W251" s="13"/>
     </row>
-    <row r="252" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="252" spans="2:23">
       <c r="B252" s="4" t="s">
         <v>113</v>
       </c>
@@ -15606,7 +15744,7 @@
       <c r="V252" s="13"/>
       <c r="W252" s="13"/>
     </row>
-    <row r="253" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="253" spans="2:23">
       <c r="B253" s="4" t="s">
         <v>114</v>
       </c>
@@ -15672,7 +15810,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="254" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="254" spans="2:23">
       <c r="B254" s="5" t="s">
         <v>8</v>
       </c>
@@ -15700,7 +15838,7 @@
       <c r="V254" s="13"/>
       <c r="W254" s="13"/>
     </row>
-    <row r="255" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="255" spans="2:23">
       <c r="B255" s="4" t="s">
         <v>115</v>
       </c>
@@ -15732,7 +15870,7 @@
       <c r="V255" s="13"/>
       <c r="W255" s="13"/>
     </row>
-    <row r="256" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="256" spans="2:23">
       <c r="B256" s="4" t="s">
         <v>116</v>
       </c>
@@ -15768,7 +15906,7 @@
       <c r="V256" s="13"/>
       <c r="W256" s="13"/>
     </row>
-    <row r="257" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="257" spans="2:23">
       <c r="B257" s="4" t="s">
         <v>117</v>
       </c>
@@ -15806,7 +15944,7 @@
       <c r="V257" s="13"/>
       <c r="W257" s="13"/>
     </row>
-    <row r="258" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="258" spans="2:23">
       <c r="B258" s="4" t="s">
         <v>118</v>
       </c>
@@ -15864,7 +16002,7 @@
       </c>
       <c r="W258" s="13"/>
     </row>
-    <row r="259" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="259" spans="2:23">
       <c r="B259" s="4" t="s">
         <v>119</v>
       </c>
@@ -15922,7 +16060,7 @@
       </c>
       <c r="W259" s="13"/>
     </row>
-    <row r="260" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="260" spans="2:23">
       <c r="B260" s="4" t="s">
         <v>120</v>
       </c>
@@ -15980,7 +16118,7 @@
       </c>
       <c r="W260" s="13"/>
     </row>
-    <row r="261" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="261" spans="2:23">
       <c r="B261" s="4" t="s">
         <v>121</v>
       </c>
@@ -16038,7 +16176,7 @@
       </c>
       <c r="W261" s="13"/>
     </row>
-    <row r="262" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="262" spans="2:23">
       <c r="B262" s="4" t="s">
         <v>122</v>
       </c>
@@ -16084,7 +16222,7 @@
       <c r="V262" s="13"/>
       <c r="W262" s="13"/>
     </row>
-    <row r="263" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="263" spans="2:23">
       <c r="B263" s="5" t="s">
         <v>8</v>
       </c>
@@ -16112,7 +16250,7 @@
       <c r="V263" s="13"/>
       <c r="W263" s="13"/>
     </row>
-    <row r="264" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="264" spans="2:23">
       <c r="B264" s="4" t="s">
         <v>123</v>
       </c>
@@ -16170,7 +16308,7 @@
       </c>
       <c r="W264" s="13"/>
     </row>
-    <row r="265" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="265" spans="2:23">
       <c r="B265" s="4" t="s">
         <v>124</v>
       </c>
@@ -16228,7 +16366,7 @@
       </c>
       <c r="W265" s="13"/>
     </row>
-    <row r="266" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="266" spans="2:23">
       <c r="B266" s="5" t="s">
         <v>8</v>
       </c>
@@ -16256,7 +16394,7 @@
       <c r="V266" s="13"/>
       <c r="W266" s="13"/>
     </row>
-    <row r="267" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="267" spans="2:23">
       <c r="B267" s="5" t="s">
         <v>125</v>
       </c>
@@ -16284,7 +16422,7 @@
       <c r="V267" s="13"/>
       <c r="W267" s="13"/>
     </row>
-    <row r="268" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="268" spans="2:23">
       <c r="B268" s="5" t="s">
         <v>125</v>
       </c>
@@ -16312,7 +16450,7 @@
       <c r="V268" s="13"/>
       <c r="W268" s="13"/>
     </row>
-    <row r="269" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="269" spans="2:23">
       <c r="B269" s="5" t="s">
         <v>125</v>
       </c>
@@ -16340,7 +16478,7 @@
       <c r="V269" s="13"/>
       <c r="W269" s="13"/>
     </row>
-    <row r="270" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="270" spans="2:23">
       <c r="B270" s="5" t="s">
         <v>125</v>
       </c>
@@ -16368,7 +16506,7 @@
       <c r="V270" s="13"/>
       <c r="W270" s="13"/>
     </row>
-    <row r="271" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="271" spans="2:23">
       <c r="B271" s="5" t="s">
         <v>125</v>
       </c>
@@ -16396,7 +16534,7 @@
       <c r="V271" s="13"/>
       <c r="W271" s="13"/>
     </row>
-    <row r="272" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="272" spans="2:23">
       <c r="B272" s="5" t="s">
         <v>125</v>
       </c>
@@ -16424,7 +16562,7 @@
       <c r="V272" s="13"/>
       <c r="W272" s="13"/>
     </row>
-    <row r="273" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="273" spans="2:23">
       <c r="B273" s="5" t="s">
         <v>125</v>
       </c>
@@ -16452,7 +16590,7 @@
       <c r="V273" s="13"/>
       <c r="W273" s="13"/>
     </row>
-    <row r="274" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="274" spans="2:23">
       <c r="B274" s="5" t="s">
         <v>125</v>
       </c>
@@ -16480,7 +16618,7 @@
       <c r="V274" s="13"/>
       <c r="W274" s="13"/>
     </row>
-    <row r="275" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="275" spans="2:23">
       <c r="B275" s="4"/>
       <c r="C275" s="3"/>
       <c r="D275" s="3"/>
@@ -16504,7 +16642,7 @@
       <c r="V275" s="13"/>
       <c r="W275" s="13"/>
     </row>
-    <row r="276" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="276" spans="2:23">
       <c r="B276" s="4"/>
       <c r="C276" s="3"/>
       <c r="D276" s="3"/>
@@ -16528,7 +16666,7 @@
       <c r="V276" s="14"/>
       <c r="W276" s="14"/>
     </row>
-    <row r="277" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="277" spans="2:23">
       <c r="B277" s="4"/>
       <c r="C277" s="3"/>
       <c r="D277" s="3"/>
@@ -16552,7 +16690,7 @@
       <c r="V277" s="14"/>
       <c r="W277" s="14"/>
     </row>
-    <row r="278" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="278" spans="2:23">
       <c r="B278" s="4"/>
       <c r="C278" s="3"/>
       <c r="D278" s="3"/>
@@ -16576,7 +16714,7 @@
       <c r="V278" s="14"/>
       <c r="W278" s="14"/>
     </row>
-    <row r="279" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="279" spans="2:23">
       <c r="B279" s="4"/>
       <c r="C279" s="3"/>
       <c r="D279" s="3"/>
@@ -16600,7 +16738,7 @@
       <c r="V279" s="14"/>
       <c r="W279" s="14"/>
     </row>
-    <row r="280" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="280" spans="2:23">
       <c r="B280" s="4"/>
       <c r="C280" s="3"/>
       <c r="D280" s="3"/>
@@ -16624,7 +16762,7 @@
       <c r="V280" s="14"/>
       <c r="W280" s="14"/>
     </row>
-    <row r="281" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="281" spans="2:23">
       <c r="B281" s="4"/>
       <c r="C281" s="3"/>
       <c r="D281" s="3"/>
@@ -16648,7 +16786,7 @@
       <c r="V281" s="14"/>
       <c r="W281" s="14"/>
     </row>
-    <row r="282" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="282" spans="2:23">
       <c r="B282" s="4"/>
       <c r="C282" s="3"/>
       <c r="D282" s="3"/>
@@ -16672,7 +16810,7 @@
       <c r="V282" s="14"/>
       <c r="W282" s="14"/>
     </row>
-    <row r="283" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="283" spans="2:23">
       <c r="B283" s="4"/>
       <c r="C283" s="3"/>
       <c r="D283" s="3"/>
@@ -16696,7 +16834,7 @@
       <c r="V283" s="14"/>
       <c r="W283" s="14"/>
     </row>
-    <row r="284" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="284" spans="2:23">
       <c r="B284" s="4"/>
       <c r="C284" s="3"/>
       <c r="D284" s="3"/>
@@ -16720,7 +16858,7 @@
       <c r="V284" s="14"/>
       <c r="W284" s="14"/>
     </row>
-    <row r="285" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="285" spans="2:23">
       <c r="B285" s="5"/>
       <c r="C285" s="17"/>
       <c r="D285" s="3"/>
@@ -16744,7 +16882,7 @@
       <c r="V285" s="14"/>
       <c r="W285" s="14"/>
     </row>
-    <row r="286" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="286" spans="2:23">
       <c r="B286" s="4"/>
       <c r="C286" s="3"/>
       <c r="D286" s="3"/>
@@ -16768,7 +16906,7 @@
       <c r="V286" s="14"/>
       <c r="W286" s="14"/>
     </row>
-    <row r="287" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="287" spans="2:23">
       <c r="B287" s="5"/>
       <c r="C287" s="17"/>
       <c r="D287" s="3"/>
@@ -16792,7 +16930,7 @@
       <c r="V287" s="14"/>
       <c r="W287" s="14"/>
     </row>
-    <row r="288" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="288" spans="2:23">
       <c r="B288" s="5"/>
       <c r="C288" s="17"/>
       <c r="D288" s="3"/>
@@ -16816,7 +16954,7 @@
       <c r="V288" s="14"/>
       <c r="W288" s="14"/>
     </row>
-    <row r="289" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="289" spans="2:23">
       <c r="B289" s="4"/>
       <c r="C289" s="3"/>
       <c r="D289" s="3"/>
@@ -16840,7 +16978,7 @@
       <c r="V289" s="14"/>
       <c r="W289" s="14"/>
     </row>
-    <row r="290" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="290" spans="2:23">
       <c r="B290" s="4"/>
       <c r="C290" s="3"/>
       <c r="D290" s="3"/>
@@ -16864,7 +17002,7 @@
       <c r="V290" s="14"/>
       <c r="W290" s="14"/>
     </row>
-    <row r="291" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="291" spans="2:23">
       <c r="B291" s="4"/>
       <c r="C291" s="3"/>
       <c r="D291" s="3"/>
@@ -16888,7 +17026,7 @@
       <c r="V291" s="14"/>
       <c r="W291" s="14"/>
     </row>
-    <row r="292" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="292" spans="2:23">
       <c r="B292" s="4"/>
       <c r="C292" s="3"/>
       <c r="D292" s="3"/>
@@ -16912,7 +17050,7 @@
       <c r="V292" s="13"/>
       <c r="W292" s="13"/>
     </row>
-    <row r="293" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="293" spans="2:23">
       <c r="B293" s="4"/>
       <c r="C293" s="3"/>
       <c r="D293" s="3"/>
@@ -16936,7 +17074,7 @@
       <c r="V293" s="14"/>
       <c r="W293" s="14"/>
     </row>
-    <row r="294" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="294" spans="2:23">
       <c r="B294" s="4"/>
       <c r="C294" s="3"/>
       <c r="D294" s="3"/>
@@ -16960,7 +17098,7 @@
       <c r="V294" s="14"/>
       <c r="W294" s="14"/>
     </row>
-    <row r="295" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="295" spans="2:23">
       <c r="B295" s="4"/>
       <c r="C295" s="3"/>
       <c r="D295" s="3"/>
@@ -16984,7 +17122,7 @@
       <c r="V295" s="14"/>
       <c r="W295" s="14"/>
     </row>
-    <row r="296" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="296" spans="2:23">
       <c r="B296" s="4"/>
       <c r="C296" s="3"/>
       <c r="D296" s="3"/>
@@ -17008,7 +17146,7 @@
       <c r="V296" s="14"/>
       <c r="W296" s="14"/>
     </row>
-    <row r="297" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="297" spans="2:23">
       <c r="B297" s="4"/>
       <c r="C297" s="3"/>
       <c r="D297" s="3"/>
@@ -17032,7 +17170,7 @@
       <c r="V297" s="14"/>
       <c r="W297" s="14"/>
     </row>
-    <row r="298" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="298" spans="2:23">
       <c r="B298" s="4"/>
       <c r="C298" s="3"/>
       <c r="D298" s="3"/>
@@ -17056,7 +17194,7 @@
       <c r="V298" s="14"/>
       <c r="W298" s="14"/>
     </row>
-    <row r="299" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="299" spans="2:23">
       <c r="B299" s="4"/>
       <c r="C299" s="3"/>
       <c r="D299" s="3"/>
@@ -17080,7 +17218,7 @@
       <c r="V299" s="14"/>
       <c r="W299" s="14"/>
     </row>
-    <row r="300" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="300" spans="2:23">
       <c r="B300" s="4"/>
       <c r="C300" s="3"/>
       <c r="D300" s="3"/>
@@ -17104,7 +17242,7 @@
       <c r="V300" s="14"/>
       <c r="W300" s="14"/>
     </row>
-    <row r="301" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="301" spans="2:23">
       <c r="B301" s="4"/>
       <c r="C301" s="3"/>
       <c r="D301" s="3"/>
@@ -17128,7 +17266,7 @@
       <c r="V301" s="14"/>
       <c r="W301" s="14"/>
     </row>
-    <row r="302" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="302" spans="2:23">
       <c r="B302" s="5"/>
       <c r="C302" s="3"/>
       <c r="D302" s="3"/>
@@ -17152,7 +17290,7 @@
       <c r="V302" s="14"/>
       <c r="W302" s="14"/>
     </row>
-    <row r="303" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="303" spans="2:23">
       <c r="B303" s="4"/>
       <c r="C303" s="3"/>
       <c r="D303" s="3"/>
@@ -17176,7 +17314,7 @@
       <c r="V303" s="14"/>
       <c r="W303" s="14"/>
     </row>
-    <row r="304" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="304" spans="2:23">
       <c r="B304" s="5"/>
       <c r="C304" s="3"/>
       <c r="D304" s="3"/>
@@ -17200,7 +17338,7 @@
       <c r="V304" s="14"/>
       <c r="W304" s="14"/>
     </row>
-    <row r="305" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="305" spans="2:23">
       <c r="B305" s="5"/>
       <c r="C305" s="3"/>
       <c r="D305" s="3"/>
@@ -17224,7 +17362,7 @@
       <c r="V305" s="14"/>
       <c r="W305" s="14"/>
     </row>
-    <row r="306" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="306" spans="2:23">
       <c r="B306" s="4"/>
       <c r="C306" s="3"/>
       <c r="D306" s="3"/>
@@ -17248,7 +17386,7 @@
       <c r="V306" s="14"/>
       <c r="W306" s="14"/>
     </row>
-    <row r="307" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="307" spans="2:23">
       <c r="B307" s="4"/>
       <c r="C307" s="3"/>
       <c r="D307" s="3"/>
@@ -17272,7 +17410,7 @@
       <c r="V307" s="14"/>
       <c r="W307" s="14"/>
     </row>
-    <row r="308" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="308" spans="2:23">
       <c r="B308" s="4"/>
       <c r="C308" s="3"/>
       <c r="D308" s="3"/>
@@ -17296,7 +17434,7 @@
       <c r="V308" s="14"/>
       <c r="W308" s="14"/>
     </row>
-    <row r="309" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="309" spans="2:23">
       <c r="B309" s="4"/>
       <c r="C309" s="3"/>
       <c r="D309" s="3"/>
@@ -17320,7 +17458,7 @@
       <c r="V309" s="13"/>
       <c r="W309" s="13"/>
     </row>
-    <row r="310" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="310" spans="2:23">
       <c r="B310" s="4"/>
       <c r="C310" s="3"/>
       <c r="D310" s="3"/>
@@ -17344,7 +17482,7 @@
       <c r="V310" s="14"/>
       <c r="W310" s="14"/>
     </row>
-    <row r="311" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="311" spans="2:23">
       <c r="B311" s="4"/>
       <c r="C311" s="3"/>
       <c r="D311" s="3"/>
@@ -17368,7 +17506,7 @@
       <c r="V311" s="14"/>
       <c r="W311" s="14"/>
     </row>
-    <row r="312" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="312" spans="2:23">
       <c r="B312" s="4"/>
       <c r="C312" s="3"/>
       <c r="D312" s="3"/>
@@ -17392,7 +17530,7 @@
       <c r="V312" s="14"/>
       <c r="W312" s="14"/>
     </row>
-    <row r="313" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="313" spans="2:23">
       <c r="B313" s="4"/>
       <c r="C313" s="3"/>
       <c r="D313" s="3"/>
@@ -17416,7 +17554,7 @@
       <c r="V313" s="14"/>
       <c r="W313" s="14"/>
     </row>
-    <row r="314" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="314" spans="2:23">
       <c r="B314" s="4"/>
       <c r="C314" s="3"/>
       <c r="D314" s="3"/>
@@ -17440,7 +17578,7 @@
       <c r="V314" s="14"/>
       <c r="W314" s="14"/>
     </row>
-    <row r="315" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="315" spans="2:23">
       <c r="B315" s="4"/>
       <c r="C315" s="3"/>
       <c r="D315" s="3"/>
@@ -17464,7 +17602,7 @@
       <c r="V315" s="14"/>
       <c r="W315" s="14"/>
     </row>
-    <row r="316" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="316" spans="2:23">
       <c r="B316" s="4"/>
       <c r="C316" s="3"/>
       <c r="D316" s="3"/>
@@ -17488,7 +17626,7 @@
       <c r="V316" s="14"/>
       <c r="W316" s="14"/>
     </row>
-    <row r="317" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="317" spans="2:23">
       <c r="B317" s="4"/>
       <c r="C317" s="3"/>
       <c r="D317" s="3"/>
@@ -17512,7 +17650,7 @@
       <c r="V317" s="14"/>
       <c r="W317" s="14"/>
     </row>
-    <row r="318" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="318" spans="2:23">
       <c r="B318" s="4"/>
       <c r="C318" s="3"/>
       <c r="D318" s="3"/>
@@ -17536,7 +17674,7 @@
       <c r="V318" s="14"/>
       <c r="W318" s="14"/>
     </row>
-    <row r="319" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="319" spans="2:23">
       <c r="B319" s="5"/>
       <c r="C319" s="3"/>
       <c r="D319" s="3"/>
@@ -17560,7 +17698,7 @@
       <c r="V319" s="14"/>
       <c r="W319" s="14"/>
     </row>
-    <row r="320" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="320" spans="2:23">
       <c r="B320" s="4"/>
       <c r="C320" s="3"/>
       <c r="D320" s="3"/>
@@ -17584,7 +17722,7 @@
       <c r="V320" s="14"/>
       <c r="W320" s="14"/>
     </row>
-    <row r="321" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="321" spans="2:23">
       <c r="B321" s="5"/>
       <c r="C321" s="3"/>
       <c r="D321" s="3"/>
@@ -17608,7 +17746,7 @@
       <c r="V321" s="14"/>
       <c r="W321" s="14"/>
     </row>
-    <row r="322" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="322" spans="2:23">
       <c r="B322" s="5"/>
       <c r="C322" s="3"/>
       <c r="D322" s="3"/>
@@ -17632,7 +17770,7 @@
       <c r="V322" s="14"/>
       <c r="W322" s="14"/>
     </row>
-    <row r="323" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="323" spans="2:23">
       <c r="B323" s="4"/>
       <c r="C323" s="3"/>
       <c r="D323" s="3"/>
@@ -17656,7 +17794,7 @@
       <c r="V323" s="14"/>
       <c r="W323" s="14"/>
     </row>
-    <row r="324" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="324" spans="2:23">
       <c r="B324" s="4"/>
       <c r="C324" s="3"/>
       <c r="D324" s="3"/>
@@ -17680,7 +17818,7 @@
       <c r="V324" s="14"/>
       <c r="W324" s="14"/>
     </row>
-    <row r="325" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="325" spans="2:23">
       <c r="B325" s="4"/>
       <c r="C325" s="3"/>
       <c r="D325" s="3"/>
@@ -17704,7 +17842,7 @@
       <c r="V325" s="14"/>
       <c r="W325" s="14"/>
     </row>
-    <row r="326" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="326" spans="2:23">
       <c r="B326" s="4"/>
       <c r="C326" s="19"/>
       <c r="D326" s="19"/>
@@ -17728,7 +17866,7 @@
       <c r="V326" s="13"/>
       <c r="W326" s="13"/>
     </row>
-    <row r="327" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="327" spans="2:23">
       <c r="B327" s="4"/>
       <c r="C327" s="3"/>
       <c r="D327" s="3"/>
@@ -17752,7 +17890,7 @@
       <c r="V327" s="14"/>
       <c r="W327" s="14"/>
     </row>
-    <row r="328" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="328" spans="2:23">
       <c r="B328" s="4"/>
       <c r="C328" s="3"/>
       <c r="D328" s="3"/>
@@ -17776,7 +17914,7 @@
       <c r="V328" s="14"/>
       <c r="W328" s="14"/>
     </row>
-    <row r="329" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="329" spans="2:23">
       <c r="B329" s="4"/>
       <c r="C329" s="3"/>
       <c r="D329" s="3"/>
@@ -17800,7 +17938,7 @@
       <c r="V329" s="14"/>
       <c r="W329" s="14"/>
     </row>
-    <row r="330" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="330" spans="2:23">
       <c r="B330" s="4"/>
       <c r="C330" s="3"/>
       <c r="D330" s="3"/>
@@ -17824,7 +17962,7 @@
       <c r="V330" s="14"/>
       <c r="W330" s="14"/>
     </row>
-    <row r="331" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="331" spans="2:23">
       <c r="B331" s="4"/>
       <c r="C331" s="3"/>
       <c r="D331" s="3"/>
@@ -17848,7 +17986,7 @@
       <c r="V331" s="14"/>
       <c r="W331" s="14"/>
     </row>
-    <row r="332" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="332" spans="2:23">
       <c r="B332" s="4"/>
       <c r="C332" s="3"/>
       <c r="D332" s="3"/>
@@ -17872,7 +18010,7 @@
       <c r="V332" s="14"/>
       <c r="W332" s="14"/>
     </row>
-    <row r="333" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="333" spans="2:23">
       <c r="B333" s="4"/>
       <c r="C333" s="3"/>
       <c r="D333" s="3"/>
@@ -17896,7 +18034,7 @@
       <c r="V333" s="14"/>
       <c r="W333" s="14"/>
     </row>
-    <row r="334" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="334" spans="2:23">
       <c r="B334" s="4"/>
       <c r="C334" s="3"/>
       <c r="D334" s="3"/>
@@ -17920,7 +18058,7 @@
       <c r="V334" s="14"/>
       <c r="W334" s="14"/>
     </row>
-    <row r="335" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="335" spans="2:23">
       <c r="B335" s="4"/>
       <c r="C335" s="3"/>
       <c r="D335" s="3"/>
@@ -17944,7 +18082,7 @@
       <c r="V335" s="14"/>
       <c r="W335" s="14"/>
     </row>
-    <row r="336" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="336" spans="2:23">
       <c r="B336" s="5"/>
       <c r="C336" s="3"/>
       <c r="D336" s="3"/>
@@ -17968,7 +18106,7 @@
       <c r="V336" s="14"/>
       <c r="W336" s="14"/>
     </row>
-    <row r="337" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="337" spans="2:23">
       <c r="B337" s="4"/>
       <c r="C337" s="3"/>
       <c r="D337" s="3"/>
@@ -17992,7 +18130,7 @@
       <c r="V337" s="14"/>
       <c r="W337" s="14"/>
     </row>
-    <row r="338" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="338" spans="2:23">
       <c r="B338" s="5"/>
       <c r="C338" s="3"/>
       <c r="D338" s="3"/>
@@ -18016,7 +18154,7 @@
       <c r="V338" s="14"/>
       <c r="W338" s="14"/>
     </row>
-    <row r="339" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="339" spans="2:23">
       <c r="B339" s="5"/>
       <c r="C339" s="3"/>
       <c r="D339" s="3"/>
@@ -18040,7 +18178,7 @@
       <c r="V339" s="14"/>
       <c r="W339" s="14"/>
     </row>
-    <row r="340" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="340" spans="2:23">
       <c r="B340" s="4"/>
       <c r="C340" s="3"/>
       <c r="D340" s="3"/>
@@ -18064,7 +18202,7 @@
       <c r="V340" s="14"/>
       <c r="W340" s="14"/>
     </row>
-    <row r="341" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="341" spans="2:23">
       <c r="B341" s="4"/>
       <c r="C341" s="3"/>
       <c r="D341" s="3"/>
@@ -18088,7 +18226,7 @@
       <c r="V341" s="14"/>
       <c r="W341" s="14"/>
     </row>
-    <row r="342" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="342" spans="2:23">
       <c r="B342" s="4"/>
       <c r="C342" s="3"/>
       <c r="D342" s="3"/>
@@ -18112,7 +18250,7 @@
       <c r="V342" s="14"/>
       <c r="W342" s="14"/>
     </row>
-    <row r="343" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="343" spans="2:23">
       <c r="B343" s="4"/>
       <c r="C343" s="3"/>
       <c r="D343" s="3"/>
@@ -18136,7 +18274,7 @@
       <c r="V343" s="14"/>
       <c r="W343" s="14"/>
     </row>
-    <row r="344" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="344" spans="2:23">
       <c r="B344" s="4"/>
       <c r="C344" s="3"/>
       <c r="D344" s="3"/>
@@ -18160,7 +18298,7 @@
       <c r="V344" s="14"/>
       <c r="W344" s="14"/>
     </row>
-    <row r="345" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="345" spans="2:23">
       <c r="B345" s="4"/>
       <c r="C345" s="3"/>
       <c r="D345" s="3"/>
@@ -18184,7 +18322,7 @@
       <c r="V345" s="14"/>
       <c r="W345" s="14"/>
     </row>
-    <row r="346" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="346" spans="2:23">
       <c r="B346" s="4"/>
       <c r="C346" s="3"/>
       <c r="D346" s="3"/>
@@ -18208,7 +18346,7 @@
       <c r="V346" s="14"/>
       <c r="W346" s="14"/>
     </row>
-    <row r="347" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="347" spans="2:23">
       <c r="B347" s="4"/>
       <c r="C347" s="3"/>
       <c r="D347" s="3"/>
@@ -18232,7 +18370,7 @@
       <c r="V347" s="14"/>
       <c r="W347" s="14"/>
     </row>
-    <row r="348" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="348" spans="2:23">
       <c r="B348" s="4"/>
       <c r="C348" s="3"/>
       <c r="D348" s="3"/>
@@ -18256,7 +18394,7 @@
       <c r="V348" s="14"/>
       <c r="W348" s="14"/>
     </row>
-    <row r="349" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="349" spans="2:23">
       <c r="B349" s="4"/>
       <c r="C349" s="3"/>
       <c r="D349" s="3"/>
@@ -18280,7 +18418,7 @@
       <c r="V349" s="14"/>
       <c r="W349" s="14"/>
     </row>
-    <row r="350" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="350" spans="2:23">
       <c r="B350" s="4"/>
       <c r="C350" s="3"/>
       <c r="D350" s="3"/>
@@ -18304,7 +18442,7 @@
       <c r="V350" s="14"/>
       <c r="W350" s="14"/>
     </row>
-    <row r="351" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="351" spans="2:23">
       <c r="B351" s="4"/>
       <c r="C351" s="19"/>
       <c r="D351" s="19"/>
@@ -18328,7 +18466,7 @@
       <c r="V351" s="13"/>
       <c r="W351" s="13"/>
     </row>
-    <row r="352" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="352" spans="2:23">
       <c r="B352" s="4" t="s">
         <v>46</v>
       </c>
@@ -18392,7 +18530,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="353" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="353" spans="2:23">
       <c r="B353" s="4" t="s">
         <v>47</v>
       </c>
@@ -18436,7 +18574,7 @@
       <c r="V353" s="13"/>
       <c r="W353" s="13"/>
     </row>
-    <row r="354" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="354" spans="2:23">
       <c r="B354" s="4" t="s">
         <v>126</v>
       </c>
@@ -18500,7 +18638,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="355" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="355" spans="2:23">
       <c r="B355" s="4" t="s">
         <v>127</v>
       </c>
@@ -18534,7 +18672,7 @@
       </c>
       <c r="W355" s="13"/>
     </row>
-    <row r="356" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="356" spans="2:23">
       <c r="B356" s="4"/>
       <c r="C356" s="3"/>
       <c r="D356" s="3"/>
@@ -18558,7 +18696,7 @@
       <c r="V356" s="13"/>
       <c r="W356" s="13"/>
     </row>
-    <row r="357" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="357" spans="2:23">
       <c r="B357" s="4" t="s">
         <v>128</v>
       </c>
@@ -18586,7 +18724,7 @@
       <c r="V357" s="13"/>
       <c r="W357" s="13"/>
     </row>
-    <row r="358" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="358" spans="2:23">
       <c r="B358" s="4" t="s">
         <v>129</v>
       </c>
@@ -18614,7 +18752,7 @@
       <c r="V358" s="13"/>
       <c r="W358" s="13"/>
     </row>
-    <row r="359" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="359" spans="2:23">
       <c r="B359" s="4" t="s">
         <v>130</v>
       </c>
@@ -18642,7 +18780,7 @@
       <c r="V359" s="13"/>
       <c r="W359" s="13"/>
     </row>
-    <row r="360" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="360" spans="2:23">
       <c r="B360" s="4" t="s">
         <v>131</v>
       </c>
@@ -18670,7 +18808,7 @@
       <c r="V360" s="13"/>
       <c r="W360" s="13"/>
     </row>
-    <row r="361" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="361" spans="2:23">
       <c r="B361" s="4" t="s">
         <v>132</v>
       </c>
@@ -18698,7 +18836,7 @@
       <c r="V361" s="13"/>
       <c r="W361" s="13"/>
     </row>
-    <row r="362" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="362" spans="2:23">
       <c r="B362" s="4"/>
       <c r="C362" s="3"/>
       <c r="D362" s="3"/>
@@ -18722,7 +18860,7 @@
       <c r="V362" s="13"/>
       <c r="W362" s="13"/>
     </row>
-    <row r="363" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="363" spans="2:23">
       <c r="B363" s="4" t="s">
         <v>128</v>
       </c>
@@ -18750,7 +18888,7 @@
       <c r="V363" s="13"/>
       <c r="W363" s="13"/>
     </row>
-    <row r="364" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="364" spans="2:23">
       <c r="B364" s="4" t="s">
         <v>129</v>
       </c>
@@ -18778,7 +18916,7 @@
       <c r="V364" s="13"/>
       <c r="W364" s="13"/>
     </row>
-    <row r="365" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="365" spans="2:23">
       <c r="B365" s="4" t="s">
         <v>130</v>
       </c>
@@ -18806,7 +18944,7 @@
       <c r="V365" s="13"/>
       <c r="W365" s="13"/>
     </row>
-    <row r="366" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="366" spans="2:23">
       <c r="B366" s="4" t="s">
         <v>131</v>
       </c>
@@ -18834,7 +18972,7 @@
       <c r="V366" s="13"/>
       <c r="W366" s="13"/>
     </row>
-    <row r="367" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="367" spans="2:23">
       <c r="B367" s="4" t="s">
         <v>132</v>
       </c>
@@ -18862,7 +19000,7 @@
       <c r="V367" s="13"/>
       <c r="W367" s="13"/>
     </row>
-    <row r="368" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="368" spans="2:23">
       <c r="B368" s="4"/>
       <c r="C368" s="3"/>
       <c r="D368" s="3"/>
@@ -18886,7 +19024,7 @@
       <c r="V368" s="13"/>
       <c r="W368" s="13"/>
     </row>
-    <row r="369" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="369" spans="2:23">
       <c r="B369" s="4" t="s">
         <v>133</v>
       </c>
@@ -18916,7 +19054,7 @@
       <c r="V369" s="13"/>
       <c r="W369" s="13"/>
     </row>
-    <row r="370" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="370" spans="2:23">
       <c r="B370" s="4" t="s">
         <v>134</v>
       </c>
@@ -18946,7 +19084,7 @@
       <c r="V370" s="13"/>
       <c r="W370" s="13"/>
     </row>
-    <row r="371" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="371" spans="2:23">
       <c r="B371" s="4" t="s">
         <v>135</v>
       </c>
@@ -18976,7 +19114,7 @@
       <c r="V371" s="13"/>
       <c r="W371" s="13"/>
     </row>
-    <row r="372" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="372" spans="2:23">
       <c r="B372" s="4"/>
       <c r="C372" s="3"/>
       <c r="D372" s="3"/>
@@ -19000,7 +19138,7 @@
       <c r="V372" s="13"/>
       <c r="W372" s="13"/>
     </row>
-    <row r="373" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="373" spans="2:23">
       <c r="B373" s="4" t="s">
         <v>133</v>
       </c>
@@ -19030,7 +19168,7 @@
       <c r="V373" s="13"/>
       <c r="W373" s="13"/>
     </row>
-    <row r="374" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="374" spans="2:23">
       <c r="B374" s="4" t="s">
         <v>134</v>
       </c>
@@ -19060,7 +19198,7 @@
       <c r="V374" s="13"/>
       <c r="W374" s="13"/>
     </row>
-    <row r="375" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="375" spans="2:23">
       <c r="B375" s="4" t="s">
         <v>135</v>
       </c>
@@ -19090,7 +19228,7 @@
       <c r="V375" s="13"/>
       <c r="W375" s="13"/>
     </row>
-    <row r="376" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="376" spans="2:23">
       <c r="B376" s="4"/>
       <c r="C376" s="3"/>
       <c r="D376" s="3"/>
@@ -19114,7 +19252,7 @@
       <c r="V376" s="13"/>
       <c r="W376" s="13"/>
     </row>
-    <row r="377" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="377" spans="2:23">
       <c r="B377" s="4"/>
       <c r="C377" s="3"/>
       <c r="D377" s="3"/>
@@ -19138,7 +19276,7 @@
       <c r="V377" s="13"/>
       <c r="W377" s="13"/>
     </row>
-    <row r="378" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="378" spans="2:23">
       <c r="B378" s="4"/>
       <c r="C378" s="3"/>
       <c r="D378" s="3"/>
@@ -19162,7 +19300,7 @@
       <c r="V378" s="13"/>
       <c r="W378" s="13"/>
     </row>
-    <row r="379" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="379" spans="2:23">
       <c r="B379" s="4"/>
       <c r="C379" s="3"/>
       <c r="D379" s="3"/>
@@ -19186,7 +19324,7 @@
       <c r="V379" s="13"/>
       <c r="W379" s="13"/>
     </row>
-    <row r="380" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="380" spans="2:23">
       <c r="B380" s="4"/>
       <c r="C380" s="3"/>
       <c r="D380" s="3"/>
@@ -19210,7 +19348,7 @@
       <c r="V380" s="13"/>
       <c r="W380" s="13"/>
     </row>
-    <row r="381" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="381" spans="2:23">
       <c r="B381" s="4"/>
       <c r="C381" s="3"/>
       <c r="D381" s="3"/>
@@ -19234,7 +19372,7 @@
       <c r="V381" s="13"/>
       <c r="W381" s="13"/>
     </row>
-    <row r="382" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="382" spans="2:23">
       <c r="B382" s="4"/>
       <c r="C382" s="3"/>
       <c r="D382" s="3"/>
@@ -19258,7 +19396,7 @@
       <c r="V382" s="13"/>
       <c r="W382" s="13"/>
     </row>
-    <row r="383" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="383" spans="2:23">
       <c r="B383" s="4"/>
       <c r="C383" s="3"/>
       <c r="D383" s="3"/>
@@ -19282,7 +19420,7 @@
       <c r="V383" s="13"/>
       <c r="W383" s="13"/>
     </row>
-    <row r="384" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="384" spans="2:23">
       <c r="B384" s="4"/>
       <c r="C384" s="3"/>
       <c r="D384" s="3"/>
@@ -19306,7 +19444,7 @@
       <c r="V384" s="13"/>
       <c r="W384" s="13"/>
     </row>
-    <row r="385" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="385" spans="2:23">
       <c r="B385" s="4"/>
       <c r="C385" s="3"/>
       <c r="D385" s="3"/>
@@ -19330,7 +19468,7 @@
       <c r="V385" s="13"/>
       <c r="W385" s="13"/>
     </row>
-    <row r="386" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="386" spans="2:23">
       <c r="B386" s="4"/>
       <c r="C386" s="3"/>
       <c r="D386" s="3"/>
@@ -19354,7 +19492,7 @@
       <c r="V386" s="13"/>
       <c r="W386" s="13"/>
     </row>
-    <row r="387" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="387" spans="2:23">
       <c r="B387" s="4"/>
       <c r="C387" s="3"/>
       <c r="D387" s="3"/>
@@ -19378,7 +19516,7 @@
       <c r="V387" s="13"/>
       <c r="W387" s="13"/>
     </row>
-    <row r="388" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="388" spans="2:23">
       <c r="B388" s="4"/>
       <c r="C388" s="3"/>
       <c r="D388" s="3"/>
@@ -19402,7 +19540,7 @@
       <c r="V388" s="13"/>
       <c r="W388" s="13"/>
     </row>
-    <row r="389" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="389" spans="2:23">
       <c r="B389" s="4"/>
       <c r="C389" s="3"/>
       <c r="D389" s="3"/>
@@ -19426,7 +19564,7 @@
       <c r="V389" s="13"/>
       <c r="W389" s="13"/>
     </row>
-    <row r="390" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="390" spans="2:23">
       <c r="B390" s="4"/>
       <c r="C390" s="3"/>
       <c r="D390" s="3"/>
@@ -19450,7 +19588,7 @@
       <c r="V390" s="13"/>
       <c r="W390" s="13"/>
     </row>
-    <row r="391" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="391" spans="2:23">
       <c r="B391" s="4"/>
       <c r="C391" s="3"/>
       <c r="D391" s="3"/>
@@ -19474,7 +19612,7 @@
       <c r="V391" s="13"/>
       <c r="W391" s="13"/>
     </row>
-    <row r="392" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="392" spans="2:23">
       <c r="B392" s="4"/>
       <c r="C392" s="3"/>
       <c r="D392" s="3"/>
@@ -19498,7 +19636,7 @@
       <c r="V392" s="13"/>
       <c r="W392" s="13"/>
     </row>
-    <row r="393" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="393" spans="2:23">
       <c r="B393" s="4"/>
       <c r="C393" s="3"/>
       <c r="D393" s="3"/>
@@ -19522,7 +19660,7 @@
       <c r="V393" s="13"/>
       <c r="W393" s="13"/>
     </row>
-    <row r="394" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="394" spans="2:23">
       <c r="B394" s="4"/>
       <c r="C394" s="3"/>
       <c r="D394" s="3"/>
@@ -19546,7 +19684,7 @@
       <c r="V394" s="13"/>
       <c r="W394" s="13"/>
     </row>
-    <row r="395" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="395" spans="2:23">
       <c r="B395" s="4"/>
       <c r="C395" s="3"/>
       <c r="D395" s="3"/>
@@ -19570,7 +19708,7 @@
       <c r="V395" s="13"/>
       <c r="W395" s="13"/>
     </row>
-    <row r="396" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="396" spans="2:23">
       <c r="B396" s="4"/>
       <c r="C396" s="3"/>
       <c r="D396" s="3"/>
@@ -19594,7 +19732,7 @@
       <c r="V396" s="13"/>
       <c r="W396" s="13"/>
     </row>
-    <row r="397" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="397" spans="2:23">
       <c r="B397" s="9"/>
       <c r="C397" s="3"/>
       <c r="D397" s="3"/>
@@ -19618,7 +19756,7 @@
       <c r="V397" s="13"/>
       <c r="W397" s="13"/>
     </row>
-    <row r="398" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="398" spans="2:23">
       <c r="B398" s="9"/>
       <c r="C398" s="3"/>
       <c r="D398" s="3"/>
@@ -19642,7 +19780,7 @@
       <c r="V398" s="13"/>
       <c r="W398" s="13"/>
     </row>
-    <row r="399" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="399" spans="2:23">
       <c r="B399" s="9"/>
       <c r="C399" s="3"/>
       <c r="D399" s="3"/>
@@ -19666,7 +19804,7 @@
       <c r="V399" s="13"/>
       <c r="W399" s="13"/>
     </row>
-    <row r="400" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="400" spans="2:23">
       <c r="B400" s="9"/>
       <c r="C400" s="3"/>
       <c r="D400" s="3"/>
@@ -19690,7 +19828,7 @@
       <c r="V400" s="13"/>
       <c r="W400" s="13"/>
     </row>
-    <row r="401" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="401" spans="2:23">
       <c r="B401" s="4"/>
       <c r="C401" s="3"/>
       <c r="D401" s="3"/>

</xml_diff>